<commit_message>
feat(nl):  add retry system
</commit_message>
<xml_diff>
--- a/Doc/ThomNardou-JDT.xlsx
+++ b/Doc/ThomNardou-JDT.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFBE1866-6C95-4990-92D5-B35253AF3373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5278B735-80B6-4285-87E8-9466BAD985EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$114</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$124</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="166">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -451,9 +451,6 @@
     <t>J'ai principalement fait de la remise en forme  mais j'ai aussi continué le résumé</t>
   </si>
   <si>
-    <t>16h10</t>
-  </si>
-  <si>
     <t>Retard</t>
   </si>
   <si>
@@ -475,9 +472,6 @@
     <t>J'ai fait quelques modification dans mon rapport et j'ai fait la video (pas fait le montage)</t>
   </si>
   <si>
-    <t>11h20</t>
-  </si>
-  <si>
     <t>Vidéo</t>
   </si>
   <si>
@@ -488,12 +482,84 @@
   </si>
   <si>
     <t>aJUSTEMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'avais donnée mon rapport à un proche pour qu'il me fasse un retour du coup je suis entrain de modifié tout cela </t>
+  </si>
+  <si>
+    <t>J'ai terminé les modifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rapport </t>
+  </si>
+  <si>
+    <t>Recherches RGPD + ajustement (~1h)</t>
+  </si>
+  <si>
+    <t>Planification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestion des rôles </t>
+  </si>
+  <si>
+    <t>Oublie</t>
+  </si>
+  <si>
+    <t>Suite à un problème (sans doute un oublie de commit) le système de renvoi n'a pas été fait ducoup j'ai du le refaire</t>
+  </si>
+  <si>
+    <t>10h10</t>
+  </si>
+  <si>
+    <t>Calcule des heures</t>
+  </si>
+  <si>
+    <t>Système d'inscription/désinscription</t>
+  </si>
+  <si>
+    <t>Interface de composition basique &amp; Interface de séléction des contact</t>
+  </si>
+  <si>
+    <t>Implémentation de la file d'attente &amp; développement du processus de relais</t>
+  </si>
+  <si>
+    <t>Système de tracking</t>
+  </si>
+  <si>
+    <t>Réalisation des tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total </t>
+  </si>
+  <si>
+    <t>Tâche non planifiées</t>
+  </si>
+  <si>
+    <t>Temps effectué</t>
+  </si>
+  <si>
+    <t>Plannifié</t>
+  </si>
+  <si>
+    <t>J'ai fait le calcule des heures pour la comparaison des heures effectuées vs planifiées</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai commencé la page de statisitique </t>
+  </si>
+  <si>
+    <t>J'ai continué la page de stats</t>
+  </si>
+  <si>
+    <t>Page de statistique</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="[h]:mm"/>
+  </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -727,7 +793,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -839,6 +905,18 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -851,12 +929,6 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -869,17 +941,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1197,7 +1272,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G157"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1213,10 +1288,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="41"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1228,10 +1303,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="41"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1243,10 +1318,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="41"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1258,12 +1333,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1286,7 +1361,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="40">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1299,7 +1374,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="39"/>
+      <c r="B7" s="41"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1312,7 +1387,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="39"/>
+      <c r="B8" s="41"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1325,7 +1400,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="39"/>
+      <c r="B9" s="41"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1336,7 +1411,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="39"/>
+      <c r="B10" s="41"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1349,7 +1424,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="39"/>
+      <c r="B11" s="41"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1364,7 +1439,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="39"/>
+      <c r="B12" s="41"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1379,7 +1454,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="39"/>
+      <c r="B13" s="41"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1394,7 +1469,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="39"/>
+      <c r="B14" s="41"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1409,9 +1484,9 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="39"/>
+      <c r="B15" s="41"/>
       <c r="C15" s="10">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>42</v>
@@ -1424,7 +1499,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="39"/>
+      <c r="B16" s="41"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1437,7 +1512,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="40"/>
+      <c r="B17" s="42"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1446,19 +1521,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="33" t="str">
+      <c r="B18" s="37" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
-        <v>5h20</v>
-      </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="35"/>
+        <v>5h25</v>
+      </c>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="39"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="38">
+      <c r="B19" s="40">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1473,7 +1548,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="39"/>
+      <c r="B20" s="41"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1486,7 +1561,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="39"/>
+      <c r="B21" s="41"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1500,7 +1575,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="39"/>
+      <c r="B22" s="41"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1513,7 +1588,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="39"/>
+      <c r="B23" s="41"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1526,7 +1601,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="39"/>
+      <c r="B24" s="41"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1539,7 +1614,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="39"/>
+      <c r="B25" s="41"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1552,7 +1627,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="39"/>
+      <c r="B26" s="41"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1565,7 +1640,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="40"/>
+      <c r="B27" s="42"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1578,19 +1653,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="33" t="str">
+      <c r="B28" s="37" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-      <c r="E28" s="35"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="39"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="38">
+      <c r="B29" s="40">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1605,7 +1680,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="39"/>
+      <c r="B30" s="41"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1620,7 +1695,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="39"/>
+      <c r="B31" s="41"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1631,14 +1706,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="39"/>
+      <c r="B32" s="41"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="40"/>
+      <c r="B33" s="42"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1647,19 +1722,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="33" t="str">
+      <c r="B34" s="37" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="34"/>
-      <c r="D34" s="34"/>
-      <c r="E34" s="35"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="39"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="38">
+      <c r="B35" s="40">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1674,7 +1749,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="39"/>
+      <c r="B36" s="41"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1687,7 +1762,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="39"/>
+      <c r="B37" s="41"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1700,7 +1775,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="39"/>
+      <c r="B38" s="41"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1713,7 +1788,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="39"/>
+      <c r="B39" s="41"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1726,7 +1801,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="39"/>
+      <c r="B40" s="41"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1739,7 +1814,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="39"/>
+      <c r="B41" s="41"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1752,7 +1827,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="39"/>
+      <c r="B42" s="41"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1765,7 +1840,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="39"/>
+      <c r="B43" s="41"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1778,7 +1853,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="40"/>
+      <c r="B44" s="42"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1791,19 +1866,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="33" t="str">
+      <c r="B45" s="37" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="34"/>
-      <c r="D45" s="34"/>
-      <c r="E45" s="35"/>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="39"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="38">
+      <c r="B46" s="40">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1818,7 +1893,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="39"/>
+      <c r="B47" s="41"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1831,7 +1906,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="39"/>
+      <c r="B48" s="41"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1844,7 +1919,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="39"/>
+      <c r="B49" s="41"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1857,7 +1932,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="39"/>
+      <c r="B50" s="41"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1870,7 +1945,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="39"/>
+      <c r="B51" s="41"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1883,9 +1958,9 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="39"/>
+      <c r="B52" s="41"/>
       <c r="C52" s="8">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>87</v>
@@ -1894,7 +1969,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="40"/>
+      <c r="B53" s="42"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1903,19 +1978,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="33" t="str">
+      <c r="B54" s="37" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
-        <v>5h20</v>
-      </c>
-      <c r="C54" s="34"/>
-      <c r="D54" s="34"/>
-      <c r="E54" s="35"/>
+        <v>5h25</v>
+      </c>
+      <c r="C54" s="38"/>
+      <c r="D54" s="38"/>
+      <c r="E54" s="39"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="38">
+      <c r="B55" s="40">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -1930,7 +2005,7 @@
       <c r="A56" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="39"/>
+      <c r="B56" s="41"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -1943,7 +2018,7 @@
       <c r="A57" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="39"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -1956,7 +2031,7 @@
       <c r="A58" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="39"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="8">
         <v>60</v>
       </c>
@@ -1969,7 +2044,7 @@
       <c r="A59" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="39"/>
+      <c r="B59" s="41"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
@@ -1982,7 +2057,7 @@
       <c r="A60" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="39"/>
+      <c r="B60" s="41"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
@@ -1995,7 +2070,7 @@
       <c r="A61" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B61" s="39"/>
+      <c r="B61" s="41"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
@@ -2008,7 +2083,7 @@
       <c r="A62" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="39"/>
+      <c r="B62" s="41"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
@@ -2021,7 +2096,7 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="39"/>
+      <c r="B63" s="41"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
@@ -2036,7 +2111,7 @@
       <c r="A64" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="39"/>
+      <c r="B64" s="41"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
@@ -2049,7 +2124,7 @@
       <c r="A65" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="39"/>
+      <c r="B65" s="41"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
@@ -2060,7 +2135,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="40"/>
+      <c r="B66" s="42"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -2069,19 +2144,19 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="33" t="str">
+      <c r="B67" s="37" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="34"/>
-      <c r="D67" s="34"/>
-      <c r="E67" s="35"/>
+      <c r="C67" s="38"/>
+      <c r="D67" s="38"/>
+      <c r="E67" s="39"/>
     </row>
     <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="38">
+      <c r="B68" s="40">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
@@ -2096,7 +2171,7 @@
       <c r="A69" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B69" s="39"/>
+      <c r="B69" s="41"/>
       <c r="C69" s="8">
         <v>60</v>
       </c>
@@ -2109,7 +2184,7 @@
       <c r="A70" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B70" s="39"/>
+      <c r="B70" s="41"/>
       <c r="C70" s="8">
         <v>55</v>
       </c>
@@ -2122,7 +2197,7 @@
       <c r="A71" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B71" s="39"/>
+      <c r="B71" s="41"/>
       <c r="C71" s="8">
         <v>15</v>
       </c>
@@ -2133,7 +2208,7 @@
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="40"/>
+      <c r="B72" s="42"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2142,19 +2217,19 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="33" t="str">
+      <c r="B73" s="37" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C73" s="34"/>
-      <c r="D73" s="34"/>
-      <c r="E73" s="35"/>
+      <c r="C73" s="38"/>
+      <c r="D73" s="38"/>
+      <c r="E73" s="39"/>
     </row>
     <row r="74" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B74" s="38">
+      <c r="B74" s="40">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
@@ -2169,7 +2244,7 @@
       <c r="A75" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="39"/>
+      <c r="B75" s="41"/>
       <c r="C75" s="8">
         <v>50</v>
       </c>
@@ -2182,7 +2257,7 @@
       <c r="A76" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="39"/>
+      <c r="B76" s="41"/>
       <c r="C76" s="8">
         <v>35</v>
       </c>
@@ -2195,7 +2270,7 @@
       <c r="A77" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B77" s="39"/>
+      <c r="B77" s="41"/>
       <c r="C77" s="8">
         <v>60</v>
       </c>
@@ -2208,7 +2283,7 @@
       <c r="A78" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B78" s="39"/>
+      <c r="B78" s="41"/>
       <c r="C78" s="10">
         <v>60</v>
       </c>
@@ -2221,7 +2296,7 @@
       <c r="A79" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B79" s="39"/>
+      <c r="B79" s="41"/>
       <c r="C79" s="10">
         <v>25</v>
       </c>
@@ -2234,7 +2309,7 @@
       <c r="A80" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B80" s="39"/>
+      <c r="B80" s="41"/>
       <c r="C80" s="10">
         <v>60</v>
       </c>
@@ -2247,7 +2322,7 @@
       <c r="A81" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="39"/>
+      <c r="B81" s="41"/>
       <c r="C81" s="10">
         <v>60</v>
       </c>
@@ -2260,7 +2335,7 @@
       <c r="A82" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B82" s="39"/>
+      <c r="B82" s="41"/>
       <c r="C82" s="10">
         <v>60</v>
       </c>
@@ -2273,7 +2348,7 @@
       <c r="A83" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B83" s="40"/>
+      <c r="B83" s="42"/>
       <c r="C83" s="10">
         <v>10</v>
       </c>
@@ -2286,19 +2361,19 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="33" t="str">
+      <c r="B84" s="37" t="str">
         <f>INT(SUM(C74:C83)/60)&amp;"h"&amp;MOD(SUM(C74:C83),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C84" s="34"/>
-      <c r="D84" s="34"/>
-      <c r="E84" s="35"/>
+      <c r="C84" s="38"/>
+      <c r="D84" s="38"/>
+      <c r="E84" s="39"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="38">
+      <c r="B85" s="40">
         <v>46153</v>
       </c>
       <c r="C85" s="5">
@@ -2313,7 +2388,7 @@
       <c r="A86" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B86" s="39"/>
+      <c r="B86" s="41"/>
       <c r="C86" s="8">
         <v>40</v>
       </c>
@@ -2326,7 +2401,7 @@
       <c r="A87" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B87" s="39"/>
+      <c r="B87" s="41"/>
       <c r="C87" s="8">
         <v>60</v>
       </c>
@@ -2339,7 +2414,7 @@
       <c r="A88" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B88" s="39"/>
+      <c r="B88" s="41"/>
       <c r="C88" s="8">
         <v>60</v>
       </c>
@@ -2352,9 +2427,9 @@
       <c r="A89" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B89" s="39"/>
+      <c r="B89" s="41"/>
       <c r="C89" s="10">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D89" s="11" t="s">
         <v>119</v>
@@ -2365,7 +2440,7 @@
       <c r="A90" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B90" s="39"/>
+      <c r="B90" s="41"/>
       <c r="C90" s="10">
         <v>60</v>
       </c>
@@ -2378,7 +2453,7 @@
       <c r="A91" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B91" s="39"/>
+      <c r="B91" s="41"/>
       <c r="C91" s="10">
         <v>60</v>
       </c>
@@ -2391,7 +2466,7 @@
       <c r="A92" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B92" s="40"/>
+      <c r="B92" s="42"/>
       <c r="C92" s="10">
         <v>10</v>
       </c>
@@ -2404,19 +2479,19 @@
       <c r="A93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B93" s="33" t="str">
+      <c r="B93" s="37" t="str">
         <f>INT(SUM(C85:C92)/60)&amp;"h"&amp;MOD(SUM(C85:C92),60)</f>
-        <v>5h20</v>
-      </c>
-      <c r="C93" s="34"/>
-      <c r="D93" s="34"/>
-      <c r="E93" s="35"/>
+        <v>5h25</v>
+      </c>
+      <c r="C93" s="38"/>
+      <c r="D93" s="38"/>
+      <c r="E93" s="39"/>
     </row>
     <row r="94" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B94" s="38">
+      <c r="B94" s="40">
         <v>46155</v>
       </c>
       <c r="C94" s="13">
@@ -2431,7 +2506,7 @@
       <c r="A95" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="39"/>
+      <c r="B95" s="41"/>
       <c r="C95" s="8">
         <v>35</v>
       </c>
@@ -2444,7 +2519,7 @@
       <c r="A96" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B96" s="39"/>
+      <c r="B96" s="41"/>
       <c r="C96" s="8">
         <v>60</v>
       </c>
@@ -2457,7 +2532,7 @@
       <c r="A97" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B97" s="39"/>
+      <c r="B97" s="41"/>
       <c r="C97" s="8">
         <v>60</v>
       </c>
@@ -2470,7 +2545,7 @@
       <c r="A98" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B98" s="39"/>
+      <c r="B98" s="41"/>
       <c r="C98" s="8">
         <v>25</v>
       </c>
@@ -2483,7 +2558,7 @@
       <c r="A99" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B99" s="39"/>
+      <c r="B99" s="41"/>
       <c r="C99" s="8">
         <v>60</v>
       </c>
@@ -2496,7 +2571,7 @@
       <c r="A100" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B100" s="39"/>
+      <c r="B100" s="41"/>
       <c r="C100" s="8">
         <v>45</v>
       </c>
@@ -2509,22 +2584,20 @@
       <c r="A101" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B101" s="39"/>
+      <c r="B101" s="41"/>
       <c r="C101" s="8">
         <v>60</v>
       </c>
       <c r="D101" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="E101" s="8" t="s">
-        <v>132</v>
-      </c>
+      <c r="E101" s="8"/>
     </row>
     <row r="102" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B102" s="40"/>
+      <c r="B102" s="42"/>
       <c r="C102" s="8">
         <v>25</v>
       </c>
@@ -2537,26 +2610,26 @@
       <c r="A103" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="33" t="str">
+      <c r="B103" s="37" t="str">
         <f>INT(SUM(C94:C102)/60)&amp;"h"&amp;MOD(SUM(C94:C102),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C103" s="34"/>
-      <c r="D103" s="34"/>
-      <c r="E103" s="35"/>
+      <c r="C103" s="38"/>
+      <c r="D103" s="38"/>
+      <c r="E103" s="39"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="B104" s="38">
+        <v>132</v>
+      </c>
+      <c r="B104" s="40">
         <v>46160</v>
       </c>
       <c r="C104" s="13">
         <v>28</v>
       </c>
       <c r="D104" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E104" s="13"/>
     </row>
@@ -2564,12 +2637,12 @@
       <c r="A105" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B105" s="39"/>
+      <c r="B105" s="41"/>
       <c r="C105" s="8">
         <v>22</v>
       </c>
       <c r="D105" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E105" s="8"/>
     </row>
@@ -2577,12 +2650,12 @@
       <c r="A106" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B106" s="39"/>
+      <c r="B106" s="41"/>
       <c r="C106" s="8">
         <v>20</v>
       </c>
       <c r="D106" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E106" s="8"/>
     </row>
@@ -2590,12 +2663,12 @@
       <c r="A107" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B107" s="39"/>
+      <c r="B107" s="41"/>
       <c r="C107" s="8">
         <v>25</v>
       </c>
       <c r="D107" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E107" s="8"/>
     </row>
@@ -2603,12 +2676,12 @@
       <c r="A108" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B108" s="39"/>
+      <c r="B108" s="41"/>
       <c r="C108" s="8">
         <v>40</v>
       </c>
       <c r="D108" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E108" s="8"/>
     </row>
@@ -2616,27 +2689,25 @@
       <c r="A109" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B109" s="39"/>
+      <c r="B109" s="41"/>
       <c r="C109" s="8">
         <v>55</v>
       </c>
       <c r="D109" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="E109" s="8" t="s">
-        <v>140</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="E109" s="8"/>
     </row>
     <row r="110" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A110" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="B110" s="39"/>
+        <v>139</v>
+      </c>
+      <c r="B110" s="41"/>
       <c r="C110" s="8">
         <v>60</v>
       </c>
       <c r="D110" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E110" s="8"/>
     </row>
@@ -2644,12 +2715,12 @@
       <c r="A111" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B111" s="39"/>
+      <c r="B111" s="41"/>
       <c r="C111" s="8">
         <v>60</v>
       </c>
       <c r="D111" s="9" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E111" s="8"/>
     </row>
@@ -2657,12 +2728,12 @@
       <c r="A112" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B112" s="40"/>
+      <c r="B112" s="42"/>
       <c r="C112" s="8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D112" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E112" s="8"/>
     </row>
@@ -2670,36 +2741,302 @@
       <c r="A113" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B113" s="33" t="str">
+      <c r="B113" s="37" t="str">
         <f>INT(SUM(C104:C112)/60)&amp;"h"&amp;MOD(SUM(C104:C112),60)</f>
-        <v>5h20</v>
-      </c>
-      <c r="C113" s="34"/>
-      <c r="D113" s="34"/>
-      <c r="E113" s="35"/>
-    </row>
-    <row r="114" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="36" t="s">
+        <v>5h25</v>
+      </c>
+      <c r="C113" s="38"/>
+      <c r="D113" s="38"/>
+      <c r="E113" s="39"/>
+    </row>
+    <row r="114" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A114" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B114" s="40">
+        <v>46162</v>
+      </c>
+      <c r="C114" s="13">
+        <v>60</v>
+      </c>
+      <c r="D114" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E114" s="13"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B115" s="41"/>
+      <c r="C115" s="8">
+        <v>35</v>
+      </c>
+      <c r="D115" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E115" s="8"/>
+    </row>
+    <row r="116" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A116" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B116" s="41"/>
+      <c r="C116" s="8">
+        <v>20</v>
+      </c>
+      <c r="D116" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B117" s="41"/>
+      <c r="C117" s="8">
+        <v>30</v>
+      </c>
+      <c r="D117" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="E117" s="8"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B118" s="41"/>
+      <c r="C118" s="8">
+        <v>60</v>
+      </c>
+      <c r="D118" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E118" s="8"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B119" s="41"/>
+      <c r="C119" s="8">
+        <v>45</v>
+      </c>
+      <c r="D119" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="E119" s="8"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" s="8"/>
+      <c r="B120" s="41"/>
+      <c r="C120" s="8"/>
+      <c r="D120" s="9"/>
+      <c r="E120" s="8"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" s="8"/>
+      <c r="B121" s="41"/>
+      <c r="C121" s="8"/>
+      <c r="D121" s="9"/>
+      <c r="E121" s="8"/>
+    </row>
+    <row r="122" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="8"/>
+      <c r="B122" s="42"/>
+      <c r="C122" s="8"/>
+      <c r="D122" s="9"/>
+      <c r="E122" s="8"/>
+    </row>
+    <row r="123" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B123" s="37" t="str">
+        <f>INT(SUM(C114:C122)/60)&amp;"h"&amp;MOD(SUM(C114:C122),60)</f>
+        <v>4h10</v>
+      </c>
+      <c r="C123" s="38"/>
+      <c r="D123" s="38"/>
+      <c r="E123" s="39"/>
+    </row>
+    <row r="124" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="B114" s="37"/>
-      <c r="C114" s="15">
-        <f>MROUND(SUM(C6:C113) /60,0.2)</f>
-        <v>63.6</v>
-      </c>
-      <c r="D114" s="16"/>
-      <c r="E114" s="17"/>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="18" t="s">
+      <c r="B124" s="44"/>
+      <c r="C124" s="15">
+        <f>MROUND(SUM(C6:C123) /60,0.2)</f>
+        <v>68</v>
+      </c>
+      <c r="D124" s="16"/>
+      <c r="E124" s="17"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="18"/>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" s="18"/>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C133" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D133" s="47" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C135" s="46">
+        <v>1.1402777777777777</v>
+      </c>
+      <c r="D135" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C137" s="24">
+        <v>6.5972222222222224E-2</v>
+      </c>
+      <c r="D137" s="24">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C139" s="24">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D139" s="24">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C141" s="24">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="D141" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C143" s="24">
+        <v>0.11458333333333333</v>
+      </c>
+      <c r="D143" s="24">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A145" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C145" s="24">
+        <v>0.15625</v>
+      </c>
+      <c r="D145" s="24">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A147" s="45" t="s">
+        <v>154</v>
+      </c>
+      <c r="C147" s="24">
+        <v>0.19791666666666666</v>
+      </c>
+      <c r="D147" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" ht="54" x14ac:dyDescent="0.25">
+      <c r="A149" s="45" t="s">
+        <v>155</v>
+      </c>
+      <c r="C149" s="24">
+        <v>0.13194444444444445</v>
+      </c>
+      <c r="D149" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C151" s="24">
+        <v>9.0277777777777776E-2</v>
+      </c>
+      <c r="D151" s="24">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C153" s="24">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D153" s="24">
+        <v>0.20833333333333334</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C155" s="46">
+        <f>C157 - SUM(C135:C153)</f>
+        <v>0.57152777777777741</v>
+      </c>
+      <c r="D155" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C157" s="46">
+        <v>2.7465277777777777</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="A124:B124"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B114:B122"/>
+    <mergeCell ref="B94:B102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B104:B112"/>
+    <mergeCell ref="B113:E113"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -2716,23 +3053,12 @@
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B113:E113"/>
-    <mergeCell ref="A114:B114"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B104:B112"/>
-    <mergeCell ref="B94:B102"/>
-    <mergeCell ref="B103:E103"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C104:C112 C19:C27 C94:C102" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C114:C122 C19:C27 C94:C102 C104:C112" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B104:B112 B94:B102" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B114:B122 B94:B102 B104:B112" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -2741,7 +3067,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="28" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="27" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -2791,7 +3117,7 @@
         <v>0.47569444444444442</v>
       </c>
       <c r="D2" s="26">
-        <v>0.51388888888888884</v>
+        <v>0.51041666666666663</v>
       </c>
       <c r="E2" s="26">
         <v>0.61458333333333337</v>
@@ -2800,7 +3126,8 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="G2" s="26">
-        <v>0.22222222222222221</v>
+        <f>C2-B2+E2-D2-F2</f>
+        <v>0.22569444444444445</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -2905,10 +3232,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E15" s="26">
-        <f>C6-B6-(F6/2)</f>
-        <v>0.16666666666666666</v>
-      </c>
+      <c r="E15" s="26"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" s="26"/>
@@ -2935,15 +3259,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -3105,6 +3420,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -3115,14 +3439,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3138,4 +3454,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(build) fix npm run build
</commit_message>
<xml_diff>
--- a/Doc/ThomNardou-JDT.xlsx
+++ b/Doc/ThomNardou-JDT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5278B735-80B6-4285-87E8-9466BAD985EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8947C979-F2C7-47AA-A54F-DCCEDDB4769B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32340" yWindow="3540" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="170">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -508,9 +508,6 @@
     <t>Suite à un problème (sans doute un oublie de commit) le système de renvoi n'a pas été fait ducoup j'ai du le refaire</t>
   </si>
   <si>
-    <t>10h10</t>
-  </si>
-  <si>
     <t>Calcule des heures</t>
   </si>
   <si>
@@ -551,6 +548,21 @@
   </si>
   <si>
     <t>Page de statistique</t>
+  </si>
+  <si>
+    <t>Divers changements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai fait quelques changement sur l'application notament la suppression du champ d'expiration du token JWT car je me suis rendu compte qu'il était inutile </t>
+  </si>
+  <si>
+    <t>14h10</t>
+  </si>
+  <si>
+    <t>Mise en production</t>
+  </si>
+  <si>
+    <t>J'ai commencé la mise ne production</t>
   </si>
 </sst>
 </file>
@@ -558,7 +570,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="[h]:mm"/>
+    <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -905,17 +917,14 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
@@ -929,6 +938,12 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -941,20 +956,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1288,10 +1300,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="44"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1303,10 +1315,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1318,10 +1330,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1333,12 +1345,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1361,7 +1373,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="40">
+      <c r="B6" s="41">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1374,7 +1386,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="41"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1387,7 +1399,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="41"/>
+      <c r="B8" s="42"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1400,7 +1412,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="41"/>
+      <c r="B9" s="42"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1411,7 +1423,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="41"/>
+      <c r="B10" s="42"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1424,7 +1436,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="41"/>
+      <c r="B11" s="42"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1439,7 +1451,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="41"/>
+      <c r="B12" s="42"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1454,7 +1466,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="41"/>
+      <c r="B13" s="42"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1469,7 +1481,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="41"/>
+      <c r="B14" s="42"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1484,7 +1496,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="41"/>
+      <c r="B15" s="42"/>
       <c r="C15" s="10">
         <v>45</v>
       </c>
@@ -1499,7 +1511,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="41"/>
+      <c r="B16" s="42"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1512,7 +1524,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="42"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1521,19 +1533,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="37" t="str">
+      <c r="B18" s="36" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="40">
+      <c r="B19" s="41">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1548,7 +1560,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="41"/>
+      <c r="B20" s="42"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1561,7 +1573,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="41"/>
+      <c r="B21" s="42"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1575,7 +1587,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="41"/>
+      <c r="B22" s="42"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1588,7 +1600,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="41"/>
+      <c r="B23" s="42"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1601,7 +1613,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="41"/>
+      <c r="B24" s="42"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1614,7 +1626,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="41"/>
+      <c r="B25" s="42"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1627,7 +1639,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="41"/>
+      <c r="B26" s="42"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1640,7 +1652,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="42"/>
+      <c r="B27" s="43"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1653,19 +1665,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="37" t="str">
+      <c r="B28" s="36" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="39"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="40">
+      <c r="B29" s="41">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1680,7 +1692,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="41"/>
+      <c r="B30" s="42"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1695,7 +1707,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="41"/>
+      <c r="B31" s="42"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1706,14 +1718,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="41"/>
+      <c r="B32" s="42"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="42"/>
+      <c r="B33" s="43"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1722,19 +1734,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="37" t="str">
+      <c r="B34" s="36" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="38"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="39"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="40">
+      <c r="B35" s="41">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1749,7 +1761,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="41"/>
+      <c r="B36" s="42"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1762,7 +1774,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="41"/>
+      <c r="B37" s="42"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1775,7 +1787,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="41"/>
+      <c r="B38" s="42"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1788,7 +1800,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="41"/>
+      <c r="B39" s="42"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1801,7 +1813,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="41"/>
+      <c r="B40" s="42"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1814,7 +1826,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="41"/>
+      <c r="B41" s="42"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1827,7 +1839,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="41"/>
+      <c r="B42" s="42"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1840,7 +1852,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="41"/>
+      <c r="B43" s="42"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1853,7 +1865,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="42"/>
+      <c r="B44" s="43"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1866,19 +1878,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="37" t="str">
+      <c r="B45" s="36" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="38"/>
-      <c r="D45" s="38"/>
-      <c r="E45" s="39"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="40">
+      <c r="B46" s="41">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1893,7 +1905,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="41"/>
+      <c r="B47" s="42"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1906,7 +1918,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="41"/>
+      <c r="B48" s="42"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1919,7 +1931,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="41"/>
+      <c r="B49" s="42"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1932,7 +1944,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="41"/>
+      <c r="B50" s="42"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1945,7 +1957,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="41"/>
+      <c r="B51" s="42"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1958,7 +1970,7 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="41"/>
+      <c r="B52" s="42"/>
       <c r="C52" s="8">
         <v>55</v>
       </c>
@@ -1969,7 +1981,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="42"/>
+      <c r="B53" s="43"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1978,19 +1990,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="37" t="str">
+      <c r="B54" s="36" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C54" s="38"/>
-      <c r="D54" s="38"/>
-      <c r="E54" s="39"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+      <c r="E54" s="38"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="40">
+      <c r="B55" s="41">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -2005,7 +2017,7 @@
       <c r="A56" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="41"/>
+      <c r="B56" s="42"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -2018,7 +2030,7 @@
       <c r="A57" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="41"/>
+      <c r="B57" s="42"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -2031,7 +2043,7 @@
       <c r="A58" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="41"/>
+      <c r="B58" s="42"/>
       <c r="C58" s="8">
         <v>60</v>
       </c>
@@ -2044,7 +2056,7 @@
       <c r="A59" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="41"/>
+      <c r="B59" s="42"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
@@ -2057,7 +2069,7 @@
       <c r="A60" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="41"/>
+      <c r="B60" s="42"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
@@ -2070,7 +2082,7 @@
       <c r="A61" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B61" s="41"/>
+      <c r="B61" s="42"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
@@ -2083,7 +2095,7 @@
       <c r="A62" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="41"/>
+      <c r="B62" s="42"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
@@ -2096,7 +2108,7 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="41"/>
+      <c r="B63" s="42"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
@@ -2111,7 +2123,7 @@
       <c r="A64" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="41"/>
+      <c r="B64" s="42"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
@@ -2124,7 +2136,7 @@
       <c r="A65" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="41"/>
+      <c r="B65" s="42"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
@@ -2135,7 +2147,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="42"/>
+      <c r="B66" s="43"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -2144,19 +2156,19 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="37" t="str">
+      <c r="B67" s="36" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="38"/>
-      <c r="D67" s="38"/>
-      <c r="E67" s="39"/>
+      <c r="C67" s="37"/>
+      <c r="D67" s="37"/>
+      <c r="E67" s="38"/>
     </row>
     <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="40">
+      <c r="B68" s="41">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
@@ -2171,7 +2183,7 @@
       <c r="A69" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B69" s="41"/>
+      <c r="B69" s="42"/>
       <c r="C69" s="8">
         <v>60</v>
       </c>
@@ -2184,7 +2196,7 @@
       <c r="A70" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B70" s="41"/>
+      <c r="B70" s="42"/>
       <c r="C70" s="8">
         <v>55</v>
       </c>
@@ -2197,7 +2209,7 @@
       <c r="A71" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B71" s="41"/>
+      <c r="B71" s="42"/>
       <c r="C71" s="8">
         <v>15</v>
       </c>
@@ -2208,7 +2220,7 @@
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="42"/>
+      <c r="B72" s="43"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2217,19 +2229,19 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="37" t="str">
+      <c r="B73" s="36" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C73" s="38"/>
-      <c r="D73" s="38"/>
-      <c r="E73" s="39"/>
+      <c r="C73" s="37"/>
+      <c r="D73" s="37"/>
+      <c r="E73" s="38"/>
     </row>
     <row r="74" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B74" s="40">
+      <c r="B74" s="41">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
@@ -2244,7 +2256,7 @@
       <c r="A75" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="41"/>
+      <c r="B75" s="42"/>
       <c r="C75" s="8">
         <v>50</v>
       </c>
@@ -2257,7 +2269,7 @@
       <c r="A76" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="41"/>
+      <c r="B76" s="42"/>
       <c r="C76" s="8">
         <v>35</v>
       </c>
@@ -2270,7 +2282,7 @@
       <c r="A77" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B77" s="41"/>
+      <c r="B77" s="42"/>
       <c r="C77" s="8">
         <v>60</v>
       </c>
@@ -2283,7 +2295,7 @@
       <c r="A78" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B78" s="41"/>
+      <c r="B78" s="42"/>
       <c r="C78" s="10">
         <v>60</v>
       </c>
@@ -2296,7 +2308,7 @@
       <c r="A79" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B79" s="41"/>
+      <c r="B79" s="42"/>
       <c r="C79" s="10">
         <v>25</v>
       </c>
@@ -2309,7 +2321,7 @@
       <c r="A80" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B80" s="41"/>
+      <c r="B80" s="42"/>
       <c r="C80" s="10">
         <v>60</v>
       </c>
@@ -2322,7 +2334,7 @@
       <c r="A81" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="41"/>
+      <c r="B81" s="42"/>
       <c r="C81" s="10">
         <v>60</v>
       </c>
@@ -2335,7 +2347,7 @@
       <c r="A82" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B82" s="41"/>
+      <c r="B82" s="42"/>
       <c r="C82" s="10">
         <v>60</v>
       </c>
@@ -2348,7 +2360,7 @@
       <c r="A83" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B83" s="42"/>
+      <c r="B83" s="43"/>
       <c r="C83" s="10">
         <v>10</v>
       </c>
@@ -2361,19 +2373,19 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="37" t="str">
+      <c r="B84" s="36" t="str">
         <f>INT(SUM(C74:C83)/60)&amp;"h"&amp;MOD(SUM(C74:C83),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C84" s="38"/>
-      <c r="D84" s="38"/>
-      <c r="E84" s="39"/>
+      <c r="C84" s="37"/>
+      <c r="D84" s="37"/>
+      <c r="E84" s="38"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="40">
+      <c r="B85" s="41">
         <v>46153</v>
       </c>
       <c r="C85" s="5">
@@ -2388,7 +2400,7 @@
       <c r="A86" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B86" s="41"/>
+      <c r="B86" s="42"/>
       <c r="C86" s="8">
         <v>40</v>
       </c>
@@ -2401,7 +2413,7 @@
       <c r="A87" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B87" s="41"/>
+      <c r="B87" s="42"/>
       <c r="C87" s="8">
         <v>60</v>
       </c>
@@ -2414,7 +2426,7 @@
       <c r="A88" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B88" s="41"/>
+      <c r="B88" s="42"/>
       <c r="C88" s="8">
         <v>60</v>
       </c>
@@ -2427,7 +2439,7 @@
       <c r="A89" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B89" s="41"/>
+      <c r="B89" s="42"/>
       <c r="C89" s="10">
         <v>15</v>
       </c>
@@ -2440,7 +2452,7 @@
       <c r="A90" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B90" s="41"/>
+      <c r="B90" s="42"/>
       <c r="C90" s="10">
         <v>60</v>
       </c>
@@ -2453,7 +2465,7 @@
       <c r="A91" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B91" s="41"/>
+      <c r="B91" s="42"/>
       <c r="C91" s="10">
         <v>60</v>
       </c>
@@ -2466,7 +2478,7 @@
       <c r="A92" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B92" s="42"/>
+      <c r="B92" s="43"/>
       <c r="C92" s="10">
         <v>10</v>
       </c>
@@ -2479,19 +2491,19 @@
       <c r="A93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B93" s="37" t="str">
+      <c r="B93" s="36" t="str">
         <f>INT(SUM(C85:C92)/60)&amp;"h"&amp;MOD(SUM(C85:C92),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C93" s="38"/>
-      <c r="D93" s="38"/>
-      <c r="E93" s="39"/>
+      <c r="C93" s="37"/>
+      <c r="D93" s="37"/>
+      <c r="E93" s="38"/>
     </row>
     <row r="94" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B94" s="40">
+      <c r="B94" s="41">
         <v>46155</v>
       </c>
       <c r="C94" s="13">
@@ -2506,7 +2518,7 @@
       <c r="A95" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="41"/>
+      <c r="B95" s="42"/>
       <c r="C95" s="8">
         <v>35</v>
       </c>
@@ -2519,7 +2531,7 @@
       <c r="A96" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B96" s="41"/>
+      <c r="B96" s="42"/>
       <c r="C96" s="8">
         <v>60</v>
       </c>
@@ -2532,7 +2544,7 @@
       <c r="A97" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B97" s="41"/>
+      <c r="B97" s="42"/>
       <c r="C97" s="8">
         <v>60</v>
       </c>
@@ -2545,7 +2557,7 @@
       <c r="A98" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B98" s="41"/>
+      <c r="B98" s="42"/>
       <c r="C98" s="8">
         <v>25</v>
       </c>
@@ -2558,7 +2570,7 @@
       <c r="A99" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B99" s="41"/>
+      <c r="B99" s="42"/>
       <c r="C99" s="8">
         <v>60</v>
       </c>
@@ -2571,7 +2583,7 @@
       <c r="A100" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B100" s="41"/>
+      <c r="B100" s="42"/>
       <c r="C100" s="8">
         <v>45</v>
       </c>
@@ -2584,7 +2596,7 @@
       <c r="A101" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B101" s="41"/>
+      <c r="B101" s="42"/>
       <c r="C101" s="8">
         <v>60</v>
       </c>
@@ -2597,7 +2609,7 @@
       <c r="A102" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B102" s="42"/>
+      <c r="B102" s="43"/>
       <c r="C102" s="8">
         <v>25</v>
       </c>
@@ -2610,19 +2622,19 @@
       <c r="A103" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="37" t="str">
+      <c r="B103" s="36" t="str">
         <f>INT(SUM(C94:C102)/60)&amp;"h"&amp;MOD(SUM(C94:C102),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C103" s="38"/>
-      <c r="D103" s="38"/>
-      <c r="E103" s="39"/>
+      <c r="C103" s="37"/>
+      <c r="D103" s="37"/>
+      <c r="E103" s="38"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B104" s="40">
+      <c r="B104" s="41">
         <v>46160</v>
       </c>
       <c r="C104" s="13">
@@ -2637,7 +2649,7 @@
       <c r="A105" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B105" s="41"/>
+      <c r="B105" s="42"/>
       <c r="C105" s="8">
         <v>22</v>
       </c>
@@ -2650,7 +2662,7 @@
       <c r="A106" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B106" s="41"/>
+      <c r="B106" s="42"/>
       <c r="C106" s="8">
         <v>20</v>
       </c>
@@ -2663,7 +2675,7 @@
       <c r="A107" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B107" s="41"/>
+      <c r="B107" s="42"/>
       <c r="C107" s="8">
         <v>25</v>
       </c>
@@ -2676,7 +2688,7 @@
       <c r="A108" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B108" s="41"/>
+      <c r="B108" s="42"/>
       <c r="C108" s="8">
         <v>40</v>
       </c>
@@ -2689,7 +2701,7 @@
       <c r="A109" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B109" s="41"/>
+      <c r="B109" s="42"/>
       <c r="C109" s="8">
         <v>55</v>
       </c>
@@ -2702,7 +2714,7 @@
       <c r="A110" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B110" s="41"/>
+      <c r="B110" s="42"/>
       <c r="C110" s="8">
         <v>60</v>
       </c>
@@ -2715,7 +2727,7 @@
       <c r="A111" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B111" s="41"/>
+      <c r="B111" s="42"/>
       <c r="C111" s="8">
         <v>60</v>
       </c>
@@ -2728,7 +2740,7 @@
       <c r="A112" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B112" s="42"/>
+      <c r="B112" s="43"/>
       <c r="C112" s="8">
         <v>15</v>
       </c>
@@ -2741,19 +2753,19 @@
       <c r="A113" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B113" s="37" t="str">
+      <c r="B113" s="36" t="str">
         <f>INT(SUM(C104:C112)/60)&amp;"h"&amp;MOD(SUM(C104:C112),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C113" s="38"/>
-      <c r="D113" s="38"/>
-      <c r="E113" s="39"/>
+      <c r="C113" s="37"/>
+      <c r="D113" s="37"/>
+      <c r="E113" s="38"/>
     </row>
     <row r="114" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A114" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B114" s="40">
+      <c r="B114" s="41">
         <v>46162</v>
       </c>
       <c r="C114" s="13">
@@ -2768,7 +2780,7 @@
       <c r="A115" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B115" s="41"/>
+      <c r="B115" s="42"/>
       <c r="C115" s="8">
         <v>35</v>
       </c>
@@ -2781,73 +2793,85 @@
       <c r="A116" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="B116" s="41"/>
+      <c r="B116" s="42"/>
       <c r="C116" s="8">
         <v>20</v>
       </c>
       <c r="D116" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="E116" s="8" t="s">
-        <v>151</v>
-      </c>
+      <c r="E116" s="8"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="B117" s="41"/>
+        <v>151</v>
+      </c>
+      <c r="B117" s="42"/>
       <c r="C117" s="8">
         <v>30</v>
       </c>
       <c r="D117" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E117" s="8"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B118" s="41"/>
+        <v>164</v>
+      </c>
+      <c r="B118" s="42"/>
       <c r="C118" s="8">
         <v>60</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E118" s="8"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B119" s="41"/>
+        <v>164</v>
+      </c>
+      <c r="B119" s="42"/>
       <c r="C119" s="8">
         <v>45</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E119" s="8"/>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A120" s="8"/>
-      <c r="B120" s="41"/>
-      <c r="C120" s="8"/>
-      <c r="D120" s="9"/>
-      <c r="E120" s="8"/>
+    <row r="120" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A120" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B120" s="42"/>
+      <c r="C120" s="8">
+        <v>60</v>
+      </c>
+      <c r="D120" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="8"/>
-      <c r="B121" s="41"/>
-      <c r="C121" s="8"/>
-      <c r="D121" s="9"/>
+      <c r="A121" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B121" s="42"/>
+      <c r="C121" s="8">
+        <v>35</v>
+      </c>
+      <c r="D121" s="9" t="s">
+        <v>169</v>
+      </c>
       <c r="E121" s="8"/>
     </row>
     <row r="122" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="8"/>
-      <c r="B122" s="42"/>
+      <c r="B122" s="43"/>
       <c r="C122" s="8"/>
       <c r="D122" s="9"/>
       <c r="E122" s="8"/>
@@ -2856,22 +2880,22 @@
       <c r="A123" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B123" s="37" t="str">
+      <c r="B123" s="36" t="str">
         <f>INT(SUM(C114:C122)/60)&amp;"h"&amp;MOD(SUM(C114:C122),60)</f>
-        <v>4h10</v>
-      </c>
-      <c r="C123" s="38"/>
-      <c r="D123" s="38"/>
-      <c r="E123" s="39"/>
+        <v>5h45</v>
+      </c>
+      <c r="C123" s="37"/>
+      <c r="D123" s="37"/>
+      <c r="E123" s="38"/>
     </row>
     <row r="124" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="43" t="s">
+      <c r="A124" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B124" s="44"/>
+      <c r="B124" s="40"/>
       <c r="C124" s="15">
         <f>MROUND(SUM(C6:C123) /60,0.2)</f>
-        <v>68</v>
+        <v>69.600000000000009</v>
       </c>
       <c r="D124" s="16"/>
       <c r="E124" s="17"/>
@@ -2886,17 +2910,17 @@
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C133" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D133" s="35" t="s">
         <v>160</v>
-      </c>
-      <c r="D133" s="47" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C135" s="46">
+      <c r="C135" s="34">
         <v>1.1402777777777777</v>
       </c>
       <c r="D135" s="24">
@@ -2949,7 +2973,7 @@
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C145" s="24">
         <v>0.15625</v>
@@ -2959,8 +2983,8 @@
       </c>
     </row>
     <row r="147" spans="1:4" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A147" s="45" t="s">
-        <v>154</v>
+      <c r="A147" s="33" t="s">
+        <v>153</v>
       </c>
       <c r="C147" s="24">
         <v>0.19791666666666666</v>
@@ -2970,8 +2994,8 @@
       </c>
     </row>
     <row r="149" spans="1:4" ht="54" x14ac:dyDescent="0.25">
-      <c r="A149" s="45" t="s">
-        <v>155</v>
+      <c r="A149" s="33" t="s">
+        <v>154</v>
       </c>
       <c r="C149" s="24">
         <v>0.13194444444444445</v>
@@ -2982,7 +3006,7 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C151" s="24">
         <v>9.0277777777777776E-2</v>
@@ -2993,7 +3017,7 @@
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C153" s="24">
         <v>8.3333333333333329E-2</v>
@@ -3004,39 +3028,26 @@
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C155" s="46">
+        <v>158</v>
+      </c>
+      <c r="C155" s="34">
         <f>C157 - SUM(C135:C153)</f>
         <v>0.57152777777777741</v>
       </c>
-      <c r="D155" s="47">
+      <c r="D155" s="35">
         <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C157" s="46">
+        <v>157</v>
+      </c>
+      <c r="C157" s="34">
         <v>2.7465277777777777</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="A124:B124"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B114:B122"/>
-    <mergeCell ref="B94:B102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B104:B112"/>
-    <mergeCell ref="B113:E113"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -3053,6 +3064,19 @@
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B55:B66"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="A124:B124"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B114:B122"/>
+    <mergeCell ref="B94:B102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B104:B112"/>
+    <mergeCell ref="B113:E113"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C114:C122 C19:C27 C94:C102 C104:C112" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -3259,6 +3283,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -3420,15 +3453,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -3439,6 +3463,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3454,12 +3486,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(app): add stats page
</commit_message>
<xml_diff>
--- a/Doc/ThomNardou-JDT.xlsx
+++ b/Doc/ThomNardou-JDT.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369D42FD-D37B-487E-8453-08DC0215B3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DA799C-CB90-442E-A706-F2623233EA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32340" yWindow="3540" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$125</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$136</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="180">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -556,9 +556,6 @@
     <t xml:space="preserve">J'ai fait quelques changement sur l'application notament la suppression du champ d'expiration du token JWT car je me suis rendu compte qu'il était inutile </t>
   </si>
   <si>
-    <t>14h10</t>
-  </si>
-  <si>
     <t>Mise en production</t>
   </si>
   <si>
@@ -572,6 +569,30 @@
   </si>
   <si>
     <t>Mise ne production terminée (problème de confiance du certificat</t>
+  </si>
+  <si>
+    <t>Disscussion</t>
+  </si>
+  <si>
+    <t>M. Melly ma envoyé un mail pour me faire un retour sur mon rapport et sur mon application et on a discuté de ce qu'il fallait modifié</t>
+  </si>
+  <si>
+    <t>Modification schémas</t>
+  </si>
+  <si>
+    <t>J'ai modifié les schémas conformément aux remarques de M. Melly</t>
+  </si>
+  <si>
+    <t>Modification Rapport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai commencé à modifier mon rapport </t>
+  </si>
+  <si>
+    <t>J'ai continué les modifications de M. Melly</t>
+  </si>
+  <si>
+    <t>J'ai presque terminé il me manque les tests manuels fait sur le serveur de staging</t>
   </si>
 </sst>
 </file>
@@ -935,6 +956,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -947,12 +980,6 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -965,17 +992,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1293,7 +1314,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G169"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1309,10 +1330,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="44"/>
+      <c r="C1" s="36"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1324,10 +1345,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="44"/>
+      <c r="C2" s="36"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1339,10 +1360,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="44"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1354,12 +1375,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="47"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1382,7 +1403,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="41">
+      <c r="B6" s="43">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1395,7 +1416,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="42"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1408,7 +1429,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="42"/>
+      <c r="B8" s="44"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1421,7 +1442,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="42"/>
+      <c r="B9" s="44"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1432,7 +1453,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="42"/>
+      <c r="B10" s="44"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1445,7 +1466,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="42"/>
+      <c r="B11" s="44"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1460,7 +1481,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="42"/>
+      <c r="B12" s="44"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1475,7 +1496,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="42"/>
+      <c r="B13" s="44"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1490,7 +1511,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="42"/>
+      <c r="B14" s="44"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1505,7 +1526,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="42"/>
+      <c r="B15" s="44"/>
       <c r="C15" s="10">
         <v>45</v>
       </c>
@@ -1520,7 +1541,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="42"/>
+      <c r="B16" s="44"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1533,7 +1554,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="43"/>
+      <c r="B17" s="45"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1542,19 +1563,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="36" t="str">
+      <c r="B18" s="40" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="42"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="41">
+      <c r="B19" s="43">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1569,7 +1590,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="42"/>
+      <c r="B20" s="44"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1582,7 +1603,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="42"/>
+      <c r="B21" s="44"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1596,7 +1617,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="42"/>
+      <c r="B22" s="44"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1609,7 +1630,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="42"/>
+      <c r="B23" s="44"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1622,7 +1643,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="42"/>
+      <c r="B24" s="44"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1635,7 +1656,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="42"/>
+      <c r="B25" s="44"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1648,7 +1669,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="42"/>
+      <c r="B26" s="44"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1661,7 +1682,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="43"/>
+      <c r="B27" s="45"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1674,19 +1695,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="36" t="str">
+      <c r="B28" s="40" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="38"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="41">
+      <c r="B29" s="43">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1701,7 +1722,7 @@
       <c r="A30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="42"/>
+      <c r="B30" s="44"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1716,7 +1737,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="42"/>
+      <c r="B31" s="44"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1727,14 +1748,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="42"/>
+      <c r="B32" s="44"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="43"/>
+      <c r="B33" s="45"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1743,19 +1764,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="36" t="str">
+      <c r="B34" s="40" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="42"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="43">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1770,7 +1791,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="42"/>
+      <c r="B36" s="44"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1783,7 +1804,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="42"/>
+      <c r="B37" s="44"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1796,7 +1817,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="42"/>
+      <c r="B38" s="44"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1809,7 +1830,7 @@
       <c r="A39" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="42"/>
+      <c r="B39" s="44"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1822,7 +1843,7 @@
       <c r="A40" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="42"/>
+      <c r="B40" s="44"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1835,7 +1856,7 @@
       <c r="A41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B41" s="42"/>
+      <c r="B41" s="44"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1848,7 +1869,7 @@
       <c r="A42" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="42"/>
+      <c r="B42" s="44"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1861,7 +1882,7 @@
       <c r="A43" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B43" s="42"/>
+      <c r="B43" s="44"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1874,7 +1895,7 @@
       <c r="A44" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="43"/>
+      <c r="B44" s="45"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1887,19 +1908,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="36" t="str">
+      <c r="B45" s="40" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="42"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B46" s="41">
+      <c r="B46" s="43">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1914,7 +1935,7 @@
       <c r="A47" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B47" s="42"/>
+      <c r="B47" s="44"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1927,7 +1948,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="42"/>
+      <c r="B48" s="44"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -1940,7 +1961,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="42"/>
+      <c r="B49" s="44"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -1953,7 +1974,7 @@
       <c r="A50" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B50" s="42"/>
+      <c r="B50" s="44"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -1966,7 +1987,7 @@
       <c r="A51" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="42"/>
+      <c r="B51" s="44"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -1979,7 +2000,7 @@
       <c r="A52" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B52" s="42"/>
+      <c r="B52" s="44"/>
       <c r="C52" s="8">
         <v>55</v>
       </c>
@@ -1990,7 +2011,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="43"/>
+      <c r="B53" s="45"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -1999,19 +2020,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="36" t="str">
+      <c r="B54" s="40" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C54" s="37"/>
-      <c r="D54" s="37"/>
-      <c r="E54" s="38"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="42"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B55" s="41">
+      <c r="B55" s="43">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -2026,7 +2047,7 @@
       <c r="A56" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="42"/>
+      <c r="B56" s="44"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -2039,7 +2060,7 @@
       <c r="A57" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="42"/>
+      <c r="B57" s="44"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -2052,7 +2073,7 @@
       <c r="A58" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="44"/>
       <c r="C58" s="8">
         <v>60</v>
       </c>
@@ -2065,7 +2086,7 @@
       <c r="A59" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="42"/>
+      <c r="B59" s="44"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
@@ -2078,7 +2099,7 @@
       <c r="A60" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="42"/>
+      <c r="B60" s="44"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
@@ -2091,7 +2112,7 @@
       <c r="A61" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B61" s="42"/>
+      <c r="B61" s="44"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
@@ -2104,7 +2125,7 @@
       <c r="A62" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="42"/>
+      <c r="B62" s="44"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
@@ -2117,7 +2138,7 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="42"/>
+      <c r="B63" s="44"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
@@ -2132,7 +2153,7 @@
       <c r="A64" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="42"/>
+      <c r="B64" s="44"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
@@ -2145,7 +2166,7 @@
       <c r="A65" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="42"/>
+      <c r="B65" s="44"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
@@ -2156,7 +2177,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="43"/>
+      <c r="B66" s="45"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -2165,19 +2186,19 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="36" t="str">
+      <c r="B67" s="40" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="37"/>
-      <c r="D67" s="37"/>
-      <c r="E67" s="38"/>
+      <c r="C67" s="41"/>
+      <c r="D67" s="41"/>
+      <c r="E67" s="42"/>
     </row>
     <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="43">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
@@ -2192,7 +2213,7 @@
       <c r="A69" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B69" s="42"/>
+      <c r="B69" s="44"/>
       <c r="C69" s="8">
         <v>60</v>
       </c>
@@ -2205,7 +2226,7 @@
       <c r="A70" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B70" s="42"/>
+      <c r="B70" s="44"/>
       <c r="C70" s="8">
         <v>55</v>
       </c>
@@ -2218,7 +2239,7 @@
       <c r="A71" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B71" s="42"/>
+      <c r="B71" s="44"/>
       <c r="C71" s="8">
         <v>15</v>
       </c>
@@ -2229,7 +2250,7 @@
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="43"/>
+      <c r="B72" s="45"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2238,19 +2259,19 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="36" t="str">
+      <c r="B73" s="40" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C73" s="37"/>
-      <c r="D73" s="37"/>
-      <c r="E73" s="38"/>
+      <c r="C73" s="41"/>
+      <c r="D73" s="41"/>
+      <c r="E73" s="42"/>
     </row>
     <row r="74" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B74" s="41">
+      <c r="B74" s="43">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
@@ -2265,7 +2286,7 @@
       <c r="A75" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="42"/>
+      <c r="B75" s="44"/>
       <c r="C75" s="8">
         <v>50</v>
       </c>
@@ -2278,7 +2299,7 @@
       <c r="A76" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="42"/>
+      <c r="B76" s="44"/>
       <c r="C76" s="8">
         <v>35</v>
       </c>
@@ -2291,7 +2312,7 @@
       <c r="A77" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B77" s="42"/>
+      <c r="B77" s="44"/>
       <c r="C77" s="8">
         <v>60</v>
       </c>
@@ -2304,7 +2325,7 @@
       <c r="A78" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B78" s="42"/>
+      <c r="B78" s="44"/>
       <c r="C78" s="10">
         <v>60</v>
       </c>
@@ -2317,7 +2338,7 @@
       <c r="A79" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B79" s="42"/>
+      <c r="B79" s="44"/>
       <c r="C79" s="10">
         <v>25</v>
       </c>
@@ -2330,7 +2351,7 @@
       <c r="A80" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B80" s="42"/>
+      <c r="B80" s="44"/>
       <c r="C80" s="10">
         <v>60</v>
       </c>
@@ -2343,7 +2364,7 @@
       <c r="A81" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="42"/>
+      <c r="B81" s="44"/>
       <c r="C81" s="10">
         <v>60</v>
       </c>
@@ -2356,7 +2377,7 @@
       <c r="A82" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B82" s="42"/>
+      <c r="B82" s="44"/>
       <c r="C82" s="10">
         <v>60</v>
       </c>
@@ -2369,7 +2390,7 @@
       <c r="A83" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B83" s="43"/>
+      <c r="B83" s="45"/>
       <c r="C83" s="10">
         <v>10</v>
       </c>
@@ -2382,19 +2403,19 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="36" t="str">
+      <c r="B84" s="40" t="str">
         <f>INT(SUM(C74:C83)/60)&amp;"h"&amp;MOD(SUM(C74:C83),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C84" s="37"/>
-      <c r="D84" s="37"/>
-      <c r="E84" s="38"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="41"/>
+      <c r="E84" s="42"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="41">
+      <c r="B85" s="43">
         <v>46153</v>
       </c>
       <c r="C85" s="5">
@@ -2409,7 +2430,7 @@
       <c r="A86" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B86" s="42"/>
+      <c r="B86" s="44"/>
       <c r="C86" s="8">
         <v>40</v>
       </c>
@@ -2422,7 +2443,7 @@
       <c r="A87" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B87" s="42"/>
+      <c r="B87" s="44"/>
       <c r="C87" s="8">
         <v>60</v>
       </c>
@@ -2435,7 +2456,7 @@
       <c r="A88" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B88" s="42"/>
+      <c r="B88" s="44"/>
       <c r="C88" s="8">
         <v>60</v>
       </c>
@@ -2448,7 +2469,7 @@
       <c r="A89" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B89" s="42"/>
+      <c r="B89" s="44"/>
       <c r="C89" s="10">
         <v>15</v>
       </c>
@@ -2461,7 +2482,7 @@
       <c r="A90" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B90" s="42"/>
+      <c r="B90" s="44"/>
       <c r="C90" s="10">
         <v>60</v>
       </c>
@@ -2474,7 +2495,7 @@
       <c r="A91" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B91" s="42"/>
+      <c r="B91" s="44"/>
       <c r="C91" s="10">
         <v>60</v>
       </c>
@@ -2487,7 +2508,7 @@
       <c r="A92" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B92" s="43"/>
+      <c r="B92" s="45"/>
       <c r="C92" s="10">
         <v>10</v>
       </c>
@@ -2500,19 +2521,19 @@
       <c r="A93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B93" s="36" t="str">
+      <c r="B93" s="40" t="str">
         <f>INT(SUM(C85:C92)/60)&amp;"h"&amp;MOD(SUM(C85:C92),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C93" s="37"/>
-      <c r="D93" s="37"/>
-      <c r="E93" s="38"/>
+      <c r="C93" s="41"/>
+      <c r="D93" s="41"/>
+      <c r="E93" s="42"/>
     </row>
     <row r="94" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B94" s="41">
+      <c r="B94" s="43">
         <v>46155</v>
       </c>
       <c r="C94" s="13">
@@ -2527,7 +2548,7 @@
       <c r="A95" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="42"/>
+      <c r="B95" s="44"/>
       <c r="C95" s="8">
         <v>35</v>
       </c>
@@ -2540,7 +2561,7 @@
       <c r="A96" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B96" s="42"/>
+      <c r="B96" s="44"/>
       <c r="C96" s="8">
         <v>60</v>
       </c>
@@ -2553,7 +2574,7 @@
       <c r="A97" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B97" s="42"/>
+      <c r="B97" s="44"/>
       <c r="C97" s="8">
         <v>60</v>
       </c>
@@ -2566,7 +2587,7 @@
       <c r="A98" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B98" s="42"/>
+      <c r="B98" s="44"/>
       <c r="C98" s="8">
         <v>25</v>
       </c>
@@ -2579,7 +2600,7 @@
       <c r="A99" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B99" s="42"/>
+      <c r="B99" s="44"/>
       <c r="C99" s="8">
         <v>60</v>
       </c>
@@ -2592,7 +2613,7 @@
       <c r="A100" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B100" s="42"/>
+      <c r="B100" s="44"/>
       <c r="C100" s="8">
         <v>45</v>
       </c>
@@ -2605,7 +2626,7 @@
       <c r="A101" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B101" s="42"/>
+      <c r="B101" s="44"/>
       <c r="C101" s="8">
         <v>60</v>
       </c>
@@ -2618,7 +2639,7 @@
       <c r="A102" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B102" s="43"/>
+      <c r="B102" s="45"/>
       <c r="C102" s="8">
         <v>25</v>
       </c>
@@ -2631,19 +2652,19 @@
       <c r="A103" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="36" t="str">
+      <c r="B103" s="40" t="str">
         <f>INT(SUM(C94:C102)/60)&amp;"h"&amp;MOD(SUM(C94:C102),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C103" s="37"/>
-      <c r="D103" s="37"/>
-      <c r="E103" s="38"/>
+      <c r="C103" s="41"/>
+      <c r="D103" s="41"/>
+      <c r="E103" s="42"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B104" s="41">
+      <c r="B104" s="43">
         <v>46160</v>
       </c>
       <c r="C104" s="13">
@@ -2658,7 +2679,7 @@
       <c r="A105" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B105" s="42"/>
+      <c r="B105" s="44"/>
       <c r="C105" s="8">
         <v>22</v>
       </c>
@@ -2671,7 +2692,7 @@
       <c r="A106" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B106" s="42"/>
+      <c r="B106" s="44"/>
       <c r="C106" s="8">
         <v>20</v>
       </c>
@@ -2684,7 +2705,7 @@
       <c r="A107" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B107" s="42"/>
+      <c r="B107" s="44"/>
       <c r="C107" s="8">
         <v>25</v>
       </c>
@@ -2697,7 +2718,7 @@
       <c r="A108" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B108" s="42"/>
+      <c r="B108" s="44"/>
       <c r="C108" s="8">
         <v>40</v>
       </c>
@@ -2710,7 +2731,7 @@
       <c r="A109" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B109" s="42"/>
+      <c r="B109" s="44"/>
       <c r="C109" s="8">
         <v>55</v>
       </c>
@@ -2723,7 +2744,7 @@
       <c r="A110" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B110" s="42"/>
+      <c r="B110" s="44"/>
       <c r="C110" s="8">
         <v>60</v>
       </c>
@@ -2736,7 +2757,7 @@
       <c r="A111" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B111" s="42"/>
+      <c r="B111" s="44"/>
       <c r="C111" s="8">
         <v>60</v>
       </c>
@@ -2749,7 +2770,7 @@
       <c r="A112" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B112" s="43"/>
+      <c r="B112" s="45"/>
       <c r="C112" s="8">
         <v>15</v>
       </c>
@@ -2762,19 +2783,19 @@
       <c r="A113" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B113" s="36" t="str">
+      <c r="B113" s="40" t="str">
         <f>INT(SUM(C104:C112)/60)&amp;"h"&amp;MOD(SUM(C104:C112),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C113" s="37"/>
-      <c r="D113" s="37"/>
-      <c r="E113" s="38"/>
+      <c r="C113" s="41"/>
+      <c r="D113" s="41"/>
+      <c r="E113" s="42"/>
     </row>
     <row r="114" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A114" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B114" s="41">
+      <c r="B114" s="43">
         <v>46162</v>
       </c>
       <c r="C114" s="13">
@@ -2789,7 +2810,7 @@
       <c r="A115" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B115" s="42"/>
+      <c r="B115" s="44"/>
       <c r="C115" s="8">
         <v>35</v>
       </c>
@@ -2802,7 +2823,7 @@
       <c r="A116" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="B116" s="42"/>
+      <c r="B116" s="44"/>
       <c r="C116" s="8">
         <v>20</v>
       </c>
@@ -2815,7 +2836,7 @@
       <c r="A117" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="B117" s="42"/>
+      <c r="B117" s="44"/>
       <c r="C117" s="8">
         <v>30</v>
       </c>
@@ -2828,7 +2849,7 @@
       <c r="A118" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="B118" s="42"/>
+      <c r="B118" s="44"/>
       <c r="C118" s="8">
         <v>60</v>
       </c>
@@ -2841,7 +2862,7 @@
       <c r="A119" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="B119" s="42"/>
+      <c r="B119" s="44"/>
       <c r="C119" s="8">
         <v>45</v>
       </c>
@@ -2854,55 +2875,51 @@
       <c r="A120" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="B120" s="42"/>
+      <c r="B120" s="44"/>
       <c r="C120" s="8">
         <v>60</v>
       </c>
       <c r="D120" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="E120" s="8" t="s">
-        <v>167</v>
-      </c>
+      <c r="E120" s="8"/>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="B121" s="42"/>
+        <v>167</v>
+      </c>
+      <c r="B121" s="44"/>
       <c r="C121" s="8">
         <v>35</v>
       </c>
       <c r="D121" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="E121" s="8" t="s">
-        <v>170</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="E121" s="8"/>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="B122" s="42"/>
+        <v>167</v>
+      </c>
+      <c r="B122" s="44"/>
       <c r="C122" s="8">
         <v>60</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E122" s="8"/>
     </row>
     <row r="123" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="B123" s="43"/>
+        <v>167</v>
+      </c>
+      <c r="B123" s="45"/>
       <c r="C123" s="8">
         <v>35</v>
       </c>
       <c r="D123" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E123" s="8"/>
     </row>
@@ -2910,174 +2927,305 @@
       <c r="A124" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B124" s="36" t="str">
+      <c r="B124" s="40" t="str">
         <f>INT(SUM(C114:C123)/60)&amp;"h"&amp;MOD(SUM(C114:C123),60)</f>
         <v>7h20</v>
       </c>
-      <c r="C124" s="37"/>
-      <c r="D124" s="37"/>
-      <c r="E124" s="38"/>
-    </row>
-    <row r="125" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A125" s="39" t="s">
+      <c r="C124" s="41"/>
+      <c r="D124" s="41"/>
+      <c r="E124" s="42"/>
+    </row>
+    <row r="125" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A125" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="B125" s="43">
+        <v>46163</v>
+      </c>
+      <c r="C125" s="13">
+        <v>30</v>
+      </c>
+      <c r="D125" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="E125" s="13"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="B126" s="44"/>
+      <c r="C126" s="8">
+        <v>30</v>
+      </c>
+      <c r="D126" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E126" s="8"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B127" s="44"/>
+      <c r="C127" s="8">
+        <v>35</v>
+      </c>
+      <c r="D127" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E127" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B128" s="44"/>
+      <c r="C128" s="8">
+        <v>60</v>
+      </c>
+      <c r="D128" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="E128" s="8"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="B129" s="44"/>
+      <c r="C129" s="8">
+        <v>35</v>
+      </c>
+      <c r="D129" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="E129" s="8"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" s="8"/>
+      <c r="B130" s="44"/>
+      <c r="C130" s="8"/>
+      <c r="D130" s="9"/>
+      <c r="E130" s="8"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" s="8"/>
+      <c r="B131" s="44"/>
+      <c r="C131" s="8"/>
+      <c r="D131" s="9"/>
+      <c r="E131" s="8"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" s="8"/>
+      <c r="B132" s="44"/>
+      <c r="C132" s="8"/>
+      <c r="D132" s="9"/>
+      <c r="E132" s="8"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" s="8"/>
+      <c r="B133" s="44"/>
+      <c r="C133" s="8"/>
+      <c r="D133" s="9"/>
+      <c r="E133" s="8"/>
+    </row>
+    <row r="134" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="8"/>
+      <c r="B134" s="45"/>
+      <c r="C134" s="8"/>
+      <c r="D134" s="9"/>
+      <c r="E134" s="8"/>
+    </row>
+    <row r="135" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B135" s="40" t="str">
+        <f>INT(SUM(C125:C134)/60)&amp;"h"&amp;MOD(SUM(C125:C134),60)</f>
+        <v>3h10</v>
+      </c>
+      <c r="C135" s="41"/>
+      <c r="D135" s="41"/>
+      <c r="E135" s="42"/>
+    </row>
+    <row r="136" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="B125" s="40"/>
-      <c r="C125" s="15">
-        <f>MROUND(SUM(C6:C124) /60,0.2)</f>
-        <v>71.2</v>
-      </c>
-      <c r="D125" s="16"/>
-      <c r="E125" s="17"/>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A127" s="18" t="s">
+      <c r="B136" s="47"/>
+      <c r="C136" s="15">
+        <f>MROUND(SUM(C6:C135) /60,0.2)</f>
+        <v>74.400000000000006</v>
+      </c>
+      <c r="D136" s="16"/>
+      <c r="E136" s="17"/>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A128" s="18"/>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C134" s="1" t="s">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" s="18"/>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C145" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D134" s="35" t="s">
+      <c r="D145" s="35" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A136" s="1" t="s">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C136" s="34">
+      <c r="C147" s="34">
         <v>1.1402777777777777</v>
       </c>
-      <c r="D136" s="24">
+      <c r="D147" s="24">
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A138" s="1" t="s">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A149" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C138" s="24">
+      <c r="C149" s="24">
         <v>6.5972222222222224E-2</v>
       </c>
-      <c r="D138" s="24">
+      <c r="D149" s="24">
         <v>0.625</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A140" s="1" t="s">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C140" s="24">
+      <c r="C151" s="24">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="D140" s="24">
+      <c r="D151" s="24">
         <v>0.125</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A142" s="1" t="s">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A153" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C142" s="24">
+      <c r="C153" s="24">
         <v>0.1111111111111111</v>
       </c>
-      <c r="D142" s="24">
+      <c r="D153" s="24">
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A144" s="1" t="s">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A155" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="C144" s="24">
+      <c r="C155" s="24">
         <v>0.11458333333333333</v>
       </c>
-      <c r="D144" s="24">
+      <c r="D155" s="24">
         <v>0.25</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A146" s="1" t="s">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C146" s="24">
+      <c r="C157" s="24">
         <v>0.15625</v>
       </c>
-      <c r="D146" s="24">
+      <c r="D157" s="24">
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A148" s="33" t="s">
+    <row r="159" spans="1:4" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A159" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="C148" s="24">
+      <c r="C159" s="24">
         <v>0.19791666666666666</v>
       </c>
-      <c r="D148" s="24">
+      <c r="D159" s="24">
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="54" x14ac:dyDescent="0.25">
-      <c r="A150" s="33" t="s">
+    <row r="161" spans="1:4" ht="54" x14ac:dyDescent="0.25">
+      <c r="A161" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="C150" s="24">
+      <c r="C161" s="24">
         <v>0.13194444444444445</v>
       </c>
-      <c r="D150" s="24">
+      <c r="D161" s="24">
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A152" s="1" t="s">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A163" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C152" s="24">
+      <c r="C163" s="24">
         <v>9.0277777777777776E-2</v>
       </c>
-      <c r="D152" s="24">
+      <c r="D163" s="24">
         <v>0.25</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A154" s="1" t="s">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A165" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C154" s="24">
+      <c r="C165" s="24">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="D154" s="24">
+      <c r="D165" s="24">
         <v>0.20833333333333334</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A156" s="1" t="s">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A167" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C156" s="34">
-        <f>C158 - SUM(C136:C154)</f>
+      <c r="C167" s="34">
+        <f>C169 - SUM(C147:C165)</f>
         <v>0.57152777777777741</v>
       </c>
-      <c r="D156" s="35">
+      <c r="D167" s="35">
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A158" s="1" t="s">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C158" s="34">
+      <c r="C169" s="34">
         <v>2.7465277777777777</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="31">
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="A136:B136"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B125:B134"/>
+    <mergeCell ref="B94:B102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B104:B112"/>
+    <mergeCell ref="B113:E113"/>
+    <mergeCell ref="B114:B123"/>
+    <mergeCell ref="B124:E124"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -3094,25 +3242,12 @@
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="A125:B125"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B114:B123"/>
-    <mergeCell ref="B94:B102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B104:B112"/>
-    <mergeCell ref="B113:E113"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C114:C123 C19:C27 C94:C102 C104:C112" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C125:C134 C19:C27 C94:C102 C104:C112 C114:C123" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B114:B123 B94:B102 B104:B112" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B125:B134 B94:B102 B104:B112 B114:B123" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -3121,7 +3256,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="27" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="25" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -3313,15 +3448,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -3483,6 +3609,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -3500,14 +3635,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3523,4 +3650,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(dashboard): move all action buttons in details page
</commit_message>
<xml_diff>
--- a/Doc/ThomNardou-JDT.xlsx
+++ b/Doc/ThomNardou-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DA799C-CB90-442E-A706-F2623233EA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03587A42-8D40-417D-9C43-2AA5CC47256F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$136</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$147</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="194">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -230,9 +230,6 @@
     <t>Ajustement</t>
   </si>
   <si>
-    <t>J'ai fait quelque ajustement au niveau de la page et j'ai aussi fait la page de politique de confidentialité (fait par IA)</t>
-  </si>
-  <si>
     <t>Inscription</t>
   </si>
   <si>
@@ -593,6 +590,51 @@
   </si>
   <si>
     <t>J'ai presque terminé il me manque les tests manuels fait sur le serveur de staging</t>
+  </si>
+  <si>
+    <t>Modification du rapport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Je suis entrain de faire mes tests manuels </t>
+  </si>
+  <si>
+    <t>J'ai continué de modifier mon rapport</t>
+  </si>
+  <si>
+    <t>Fix gestion d'erreur script</t>
+  </si>
+  <si>
+    <t>J'ai rmarqué un bug ou le script essayais de d'envoyer la meme campagne en boucle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai terminé de fix le problème si j'ai pris beaucoup de temps c'est parce que j'ai voulu m'aidé de l'IA pour le reglé rapidement mais au final elle me donnait que des choses fausse donc j'en ai eu marre et j'ai corrigé le bug moi-même (que ca me serve de leçon) et au final c'est juste qu'il traitait les lecteur plusieur fois même si l'envoi avait échoué ducoup j'ai rajouté un champ en db pour évité qu'il soit repris en compte </t>
+  </si>
+  <si>
+    <t>J'ai continué mon rapport là je vais faire le première version de la comparaison du temps plannifié et effectué</t>
+  </si>
+  <si>
+    <t>Journal de travail</t>
+  </si>
+  <si>
+    <t>Rapport Plannification</t>
+  </si>
+  <si>
+    <t>J'ai fait quelque ajustement au niveau de la page d'inscription et j'ai aussi fait la page de politique de confidentialité (fait par IA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai essayé d'améliorer la vidéo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modification détails d'une campagne </t>
+  </si>
+  <si>
+    <t>Suite à plusieurs demandes de M. j'ai commencé à modifier l'app</t>
+  </si>
+  <si>
+    <t>Correction système de suppression</t>
+  </si>
+  <si>
+    <t>J'ai commencé à modifier le système de suppression</t>
   </si>
 </sst>
 </file>
@@ -835,7 +877,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -956,18 +998,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -980,6 +1010,12 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -992,11 +1028,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1314,7 +1359,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G169"/>
+  <dimension ref="A1:G180"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1330,10 +1375,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="36"/>
+      <c r="C1" s="44"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1345,10 +1390,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="36"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1360,10 +1405,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="36"/>
+      <c r="C3" s="44"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1375,12 +1420,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1403,7 +1448,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="43">
+      <c r="B6" s="41">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1416,7 +1461,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="44"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1429,7 +1474,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="44"/>
+      <c r="B8" s="42"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1442,7 +1487,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="44"/>
+      <c r="B9" s="42"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1453,7 +1498,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="44"/>
+      <c r="B10" s="42"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1466,7 +1511,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="44"/>
+      <c r="B11" s="42"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1481,7 +1526,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="44"/>
+      <c r="B12" s="42"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1496,7 +1541,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="44"/>
+      <c r="B13" s="42"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1511,7 +1556,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="44"/>
+      <c r="B14" s="42"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1526,7 +1571,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="44"/>
+      <c r="B15" s="42"/>
       <c r="C15" s="10">
         <v>45</v>
       </c>
@@ -1541,7 +1586,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="44"/>
+      <c r="B16" s="42"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1554,7 +1599,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="45"/>
+      <c r="B17" s="43"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1563,19 +1608,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="40" t="str">
+      <c r="B18" s="36" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="42"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="38"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="43">
+      <c r="B19" s="41">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1590,7 +1635,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="44"/>
+      <c r="B20" s="42"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1603,7 +1648,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="44"/>
+      <c r="B21" s="42"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1617,7 +1662,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="44"/>
+      <c r="B22" s="42"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1630,7 +1675,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="44"/>
+      <c r="B23" s="42"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1643,7 +1688,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="44"/>
+      <c r="B24" s="42"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1656,7 +1701,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="44"/>
+      <c r="B25" s="42"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1669,7 +1714,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="44"/>
+      <c r="B26" s="42"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1682,12 +1727,12 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="45"/>
+      <c r="B27" s="43"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>59</v>
+        <v>188</v>
       </c>
       <c r="E27" s="10"/>
     </row>
@@ -1695,67 +1740,67 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="40" t="str">
+      <c r="B28" s="36" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="41"/>
-      <c r="D28" s="41"/>
-      <c r="E28" s="42"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="38"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B29" s="43">
+        <v>59</v>
+      </c>
+      <c r="B29" s="41">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
         <v>60</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E29" s="5"/>
     </row>
     <row r="30" spans="1:7" ht="54" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="42"/>
+      <c r="C30" s="8">
+        <v>60</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B30" s="44"/>
-      <c r="C30" s="8">
-        <v>60</v>
-      </c>
-      <c r="D30" s="9" t="s">
+      <c r="E30" s="27" t="s">
         <v>63</v>
-      </c>
-      <c r="E30" s="27" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="27" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="44"/>
+      <c r="B31" s="42"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="44"/>
+      <c r="B32" s="42"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="45"/>
+      <c r="B33" s="43"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1764,26 +1809,26 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="40" t="str">
+      <c r="B34" s="36" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="41"/>
-      <c r="D34" s="41"/>
-      <c r="E34" s="42"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="38"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="43">
+      <c r="B35" s="41">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
         <v>60</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E35" s="5"/>
     </row>
@@ -1791,12 +1836,12 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="44"/>
+      <c r="B36" s="42"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E36" s="8"/>
     </row>
@@ -1804,12 +1849,12 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="44"/>
+      <c r="B37" s="42"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E37" s="8"/>
     </row>
@@ -1817,90 +1862,90 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="44"/>
+      <c r="B38" s="42"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="B39" s="44"/>
+        <v>69</v>
+      </c>
+      <c r="B39" s="42"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="B40" s="44"/>
+        <v>71</v>
+      </c>
+      <c r="B40" s="42"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="B41" s="44"/>
+        <v>71</v>
+      </c>
+      <c r="B41" s="42"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="B42" s="44"/>
+        <v>71</v>
+      </c>
+      <c r="B42" s="42"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="B43" s="42"/>
+      <c r="C43" s="10">
+        <v>60</v>
+      </c>
+      <c r="D43" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="B43" s="44"/>
-      <c r="C43" s="10">
-        <v>60</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>77</v>
       </c>
       <c r="E43" s="29"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="B44" s="45"/>
+        <v>75</v>
+      </c>
+      <c r="B44" s="43"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
       <c r="D44" s="30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E44" s="29"/>
     </row>
@@ -1908,39 +1953,39 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="40" t="str">
+      <c r="B45" s="36" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="41"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="42"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="37"/>
+      <c r="E45" s="38"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="B46" s="43">
+        <v>75</v>
+      </c>
+      <c r="B46" s="41">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
         <v>50</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E46" s="13"/>
     </row>
     <row r="47" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B47" s="44"/>
+        <v>75</v>
+      </c>
+      <c r="B47" s="42"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E47" s="31"/>
     </row>
@@ -1948,12 +1993,12 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="44"/>
+      <c r="B48" s="42"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E48" s="31"/>
     </row>
@@ -1961,57 +2006,57 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="44"/>
+      <c r="B49" s="42"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E49" s="31"/>
     </row>
     <row r="50" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A50" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B50" s="42"/>
+      <c r="C50" s="8">
+        <v>60</v>
+      </c>
+      <c r="D50" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="B50" s="44"/>
-      <c r="C50" s="8">
-        <v>60</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>84</v>
       </c>
       <c r="E50" s="31"/>
     </row>
     <row r="51" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B51" s="44"/>
+        <v>82</v>
+      </c>
+      <c r="B51" s="42"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E51" s="31"/>
     </row>
     <row r="52" spans="1:5" ht="108" x14ac:dyDescent="0.25">
       <c r="A52" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="B52" s="44"/>
+        <v>85</v>
+      </c>
+      <c r="B52" s="42"/>
       <c r="C52" s="8">
         <v>55</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E52" s="31"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="45"/>
+      <c r="B53" s="43"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -2020,117 +2065,117 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="40" t="str">
+      <c r="B54" s="36" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C54" s="41"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="42"/>
+      <c r="C54" s="37"/>
+      <c r="D54" s="37"/>
+      <c r="E54" s="38"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B55" s="41">
+        <v>46148</v>
+      </c>
+      <c r="C55" s="5">
+        <v>60</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="B55" s="43">
-        <v>46148</v>
-      </c>
-      <c r="C55" s="5">
-        <v>60</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="E55" s="5"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B56" s="44"/>
+        <v>89</v>
+      </c>
+      <c r="B56" s="42"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B57" s="44"/>
+        <v>89</v>
+      </c>
+      <c r="B57" s="42"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B58" s="42"/>
+      <c r="C58" s="8">
+        <v>60</v>
+      </c>
+      <c r="D58" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="B58" s="44"/>
-      <c r="C58" s="8">
-        <v>60</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="B59" s="44"/>
+        <v>94</v>
+      </c>
+      <c r="B59" s="42"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
       <c r="D59" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="B60" s="44"/>
+        <v>94</v>
+      </c>
+      <c r="B60" s="42"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
       <c r="D60" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="B61" s="44"/>
+        <v>97</v>
+      </c>
+      <c r="B61" s="42"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
       <c r="D61" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="B62" s="44"/>
+        <v>94</v>
+      </c>
+      <c r="B62" s="42"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
       <c r="D62" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E62" s="10"/>
     </row>
@@ -2138,46 +2183,46 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="44"/>
+      <c r="B63" s="42"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
       <c r="D63" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E63" s="10" t="s">
         <v>101</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="B64" s="44"/>
+        <v>187</v>
+      </c>
+      <c r="B64" s="42"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
       <c r="D64" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A65" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="B65" s="44"/>
+        <v>187</v>
+      </c>
+      <c r="B65" s="42"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="45"/>
+      <c r="B66" s="43"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -2186,52 +2231,52 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="40" t="str">
+      <c r="B67" s="36" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="41"/>
-      <c r="D67" s="41"/>
-      <c r="E67" s="42"/>
+      <c r="C67" s="37"/>
+      <c r="D67" s="37"/>
+      <c r="E67" s="38"/>
     </row>
     <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="43">
+      <c r="B68" s="41">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
         <v>60</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E68" s="5"/>
     </row>
     <row r="69" spans="1:5" ht="54" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B69" s="42"/>
+      <c r="C69" s="8">
+        <v>60</v>
+      </c>
+      <c r="D69" s="9" t="s">
         <v>106</v>
-      </c>
-      <c r="B69" s="44"/>
-      <c r="C69" s="8">
-        <v>60</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>107</v>
       </c>
       <c r="E69" s="8"/>
     </row>
     <row r="70" spans="1:5" ht="81" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="B70" s="44"/>
+        <v>107</v>
+      </c>
+      <c r="B70" s="42"/>
       <c r="C70" s="8">
         <v>55</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E70" s="8"/>
     </row>
@@ -2239,18 +2284,18 @@
       <c r="A71" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B71" s="44"/>
+      <c r="B71" s="42"/>
       <c r="C71" s="8">
         <v>15</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="45"/>
+      <c r="B72" s="43"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2259,26 +2304,26 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="40" t="str">
+      <c r="B73" s="36" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C73" s="41"/>
-      <c r="D73" s="41"/>
-      <c r="E73" s="42"/>
+      <c r="C73" s="37"/>
+      <c r="D73" s="37"/>
+      <c r="E73" s="38"/>
     </row>
     <row r="74" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B74" s="43">
+        <v>92</v>
+      </c>
+      <c r="B74" s="41">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
         <v>10</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E74" s="5"/>
     </row>
@@ -2286,12 +2331,12 @@
       <c r="A75" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="44"/>
+      <c r="B75" s="42"/>
       <c r="C75" s="8">
         <v>50</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E75" s="8"/>
     </row>
@@ -2299,38 +2344,38 @@
       <c r="A76" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="44"/>
+      <c r="B76" s="42"/>
       <c r="C76" s="8">
         <v>35</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B77" s="42"/>
+      <c r="C77" s="8">
+        <v>60</v>
+      </c>
+      <c r="D77" s="9" t="s">
         <v>114</v>
-      </c>
-      <c r="B77" s="44"/>
-      <c r="C77" s="8">
-        <v>60</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>115</v>
       </c>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="B78" s="44"/>
+        <v>113</v>
+      </c>
+      <c r="B78" s="42"/>
       <c r="C78" s="10">
         <v>60</v>
       </c>
       <c r="D78" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E78" s="10"/>
     </row>
@@ -2338,12 +2383,12 @@
       <c r="A79" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B79" s="44"/>
+      <c r="B79" s="42"/>
       <c r="C79" s="10">
         <v>25</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E79" s="10"/>
     </row>
@@ -2351,12 +2396,12 @@
       <c r="A80" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B80" s="44"/>
+      <c r="B80" s="42"/>
       <c r="C80" s="10">
         <v>60</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E80" s="10"/>
     </row>
@@ -2364,12 +2409,12 @@
       <c r="A81" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="44"/>
+      <c r="B81" s="42"/>
       <c r="C81" s="10">
         <v>60</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E81" s="10"/>
     </row>
@@ -2377,12 +2422,12 @@
       <c r="A82" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B82" s="44"/>
+      <c r="B82" s="42"/>
       <c r="C82" s="10">
         <v>60</v>
       </c>
       <c r="D82" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E82" s="10"/>
     </row>
@@ -2390,12 +2435,12 @@
       <c r="A83" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B83" s="45"/>
+      <c r="B83" s="43"/>
       <c r="C83" s="10">
         <v>10</v>
       </c>
       <c r="D83" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E83" s="10"/>
     </row>
@@ -2403,39 +2448,39 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="40" t="str">
+      <c r="B84" s="36" t="str">
         <f>INT(SUM(C74:C83)/60)&amp;"h"&amp;MOD(SUM(C74:C83),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C84" s="41"/>
-      <c r="D84" s="41"/>
-      <c r="E84" s="42"/>
+      <c r="C84" s="37"/>
+      <c r="D84" s="37"/>
+      <c r="E84" s="38"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="43">
+      <c r="B85" s="41">
         <v>46153</v>
       </c>
       <c r="C85" s="5">
         <v>20</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E85" s="5"/>
     </row>
     <row r="86" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="B86" s="44"/>
+        <v>120</v>
+      </c>
+      <c r="B86" s="42"/>
       <c r="C86" s="8">
         <v>40</v>
       </c>
       <c r="D86" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E86" s="8"/>
     </row>
@@ -2443,12 +2488,12 @@
       <c r="A87" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B87" s="44"/>
+      <c r="B87" s="42"/>
       <c r="C87" s="8">
         <v>60</v>
       </c>
       <c r="D87" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E87" s="8"/>
     </row>
@@ -2456,12 +2501,12 @@
       <c r="A88" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B88" s="44"/>
+      <c r="B88" s="42"/>
       <c r="C88" s="8">
         <v>60</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E88" s="8"/>
     </row>
@@ -2469,12 +2514,12 @@
       <c r="A89" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B89" s="44"/>
+      <c r="B89" s="42"/>
       <c r="C89" s="10">
         <v>15</v>
       </c>
       <c r="D89" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E89" s="10"/>
     </row>
@@ -2482,12 +2527,12 @@
       <c r="A90" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B90" s="44"/>
+      <c r="B90" s="42"/>
       <c r="C90" s="10">
         <v>60</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E90" s="10"/>
     </row>
@@ -2495,12 +2540,12 @@
       <c r="A91" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B91" s="44"/>
+      <c r="B91" s="42"/>
       <c r="C91" s="10">
         <v>60</v>
       </c>
       <c r="D91" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E91" s="10"/>
     </row>
@@ -2508,12 +2553,12 @@
       <c r="A92" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B92" s="45"/>
+      <c r="B92" s="43"/>
       <c r="C92" s="10">
         <v>10</v>
       </c>
       <c r="D92" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E92" s="10"/>
     </row>
@@ -2521,26 +2566,26 @@
       <c r="A93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B93" s="40" t="str">
+      <c r="B93" s="36" t="str">
         <f>INT(SUM(C85:C92)/60)&amp;"h"&amp;MOD(SUM(C85:C92),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C93" s="41"/>
-      <c r="D93" s="41"/>
-      <c r="E93" s="42"/>
+      <c r="C93" s="37"/>
+      <c r="D93" s="37"/>
+      <c r="E93" s="38"/>
     </row>
     <row r="94" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B94" s="43">
+      <c r="B94" s="41">
         <v>46155</v>
       </c>
       <c r="C94" s="13">
         <v>60</v>
       </c>
       <c r="D94" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E94" s="13"/>
     </row>
@@ -2548,12 +2593,12 @@
       <c r="A95" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="44"/>
+      <c r="B95" s="42"/>
       <c r="C95" s="8">
         <v>35</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E95" s="8"/>
     </row>
@@ -2561,12 +2606,12 @@
       <c r="A96" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B96" s="44"/>
+      <c r="B96" s="42"/>
       <c r="C96" s="8">
         <v>60</v>
       </c>
       <c r="D96" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E96" s="8"/>
     </row>
@@ -2574,12 +2619,12 @@
       <c r="A97" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B97" s="44"/>
+      <c r="B97" s="42"/>
       <c r="C97" s="8">
         <v>60</v>
       </c>
       <c r="D97" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E97" s="8"/>
     </row>
@@ -2587,12 +2632,12 @@
       <c r="A98" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B98" s="44"/>
+      <c r="B98" s="42"/>
       <c r="C98" s="8">
         <v>25</v>
       </c>
       <c r="D98" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E98" s="8"/>
     </row>
@@ -2600,12 +2645,12 @@
       <c r="A99" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B99" s="44"/>
+      <c r="B99" s="42"/>
       <c r="C99" s="8">
         <v>60</v>
       </c>
       <c r="D99" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E99" s="8"/>
     </row>
@@ -2613,12 +2658,12 @@
       <c r="A100" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B100" s="44"/>
+      <c r="B100" s="42"/>
       <c r="C100" s="8">
         <v>45</v>
       </c>
       <c r="D100" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E100" s="8"/>
     </row>
@@ -2626,12 +2671,12 @@
       <c r="A101" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B101" s="44"/>
+      <c r="B101" s="42"/>
       <c r="C101" s="8">
         <v>60</v>
       </c>
       <c r="D101" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E101" s="8"/>
     </row>
@@ -2639,12 +2684,12 @@
       <c r="A102" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B102" s="45"/>
+      <c r="B102" s="43"/>
       <c r="C102" s="8">
         <v>25</v>
       </c>
       <c r="D102" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E102" s="8"/>
     </row>
@@ -2652,26 +2697,26 @@
       <c r="A103" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="40" t="str">
+      <c r="B103" s="36" t="str">
         <f>INT(SUM(C94:C102)/60)&amp;"h"&amp;MOD(SUM(C94:C102),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C103" s="41"/>
-      <c r="D103" s="41"/>
-      <c r="E103" s="42"/>
+      <c r="C103" s="37"/>
+      <c r="D103" s="37"/>
+      <c r="E103" s="38"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="B104" s="43">
+        <v>131</v>
+      </c>
+      <c r="B104" s="41">
         <v>46160</v>
       </c>
       <c r="C104" s="13">
         <v>28</v>
       </c>
       <c r="D104" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E104" s="13"/>
     </row>
@@ -2679,12 +2724,12 @@
       <c r="A105" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B105" s="44"/>
+      <c r="B105" s="42"/>
       <c r="C105" s="8">
         <v>22</v>
       </c>
       <c r="D105" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E105" s="8"/>
     </row>
@@ -2692,12 +2737,12 @@
       <c r="A106" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B106" s="44"/>
+      <c r="B106" s="42"/>
       <c r="C106" s="8">
         <v>20</v>
       </c>
       <c r="D106" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E106" s="8"/>
     </row>
@@ -2705,12 +2750,12 @@
       <c r="A107" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B107" s="44"/>
+      <c r="B107" s="42"/>
       <c r="C107" s="8">
         <v>25</v>
       </c>
       <c r="D107" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E107" s="8"/>
     </row>
@@ -2718,12 +2763,12 @@
       <c r="A108" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B108" s="44"/>
+      <c r="B108" s="42"/>
       <c r="C108" s="8">
         <v>40</v>
       </c>
       <c r="D108" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E108" s="8"/>
     </row>
@@ -2731,25 +2776,25 @@
       <c r="A109" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B109" s="44"/>
+      <c r="B109" s="42"/>
       <c r="C109" s="8">
         <v>55</v>
       </c>
       <c r="D109" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E109" s="8"/>
     </row>
     <row r="110" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A110" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B110" s="42"/>
+      <c r="C110" s="8">
+        <v>60</v>
+      </c>
+      <c r="D110" s="9" t="s">
         <v>139</v>
-      </c>
-      <c r="B110" s="44"/>
-      <c r="C110" s="8">
-        <v>60</v>
-      </c>
-      <c r="D110" s="9" t="s">
-        <v>140</v>
       </c>
       <c r="E110" s="8"/>
     </row>
@@ -2757,12 +2802,12 @@
       <c r="A111" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B111" s="44"/>
+      <c r="B111" s="42"/>
       <c r="C111" s="8">
         <v>60</v>
       </c>
       <c r="D111" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E111" s="8"/>
     </row>
@@ -2770,12 +2815,12 @@
       <c r="A112" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B112" s="45"/>
+      <c r="B112" s="43"/>
       <c r="C112" s="8">
         <v>15</v>
       </c>
       <c r="D112" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E112" s="8"/>
     </row>
@@ -2783,26 +2828,26 @@
       <c r="A113" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B113" s="40" t="str">
+      <c r="B113" s="36" t="str">
         <f>INT(SUM(C104:C112)/60)&amp;"h"&amp;MOD(SUM(C104:C112),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C113" s="41"/>
-      <c r="D113" s="41"/>
-      <c r="E113" s="42"/>
+      <c r="C113" s="37"/>
+      <c r="D113" s="37"/>
+      <c r="E113" s="38"/>
     </row>
     <row r="114" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A114" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B114" s="43">
+      <c r="B114" s="41">
         <v>46162</v>
       </c>
       <c r="C114" s="13">
         <v>60</v>
       </c>
       <c r="D114" s="14" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E114" s="13"/>
     </row>
@@ -2810,116 +2855,116 @@
       <c r="A115" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B115" s="44"/>
+      <c r="B115" s="42"/>
       <c r="C115" s="8">
         <v>35</v>
       </c>
       <c r="D115" s="9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E115" s="8"/>
     </row>
     <row r="116" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A116" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B116" s="44"/>
+        <v>148</v>
+      </c>
+      <c r="B116" s="42"/>
       <c r="C116" s="8">
         <v>20</v>
       </c>
       <c r="D116" s="9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E116" s="8"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="B117" s="44"/>
+        <v>150</v>
+      </c>
+      <c r="B117" s="42"/>
       <c r="C117" s="8">
         <v>30</v>
       </c>
       <c r="D117" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E117" s="8"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B118" s="44"/>
+        <v>163</v>
+      </c>
+      <c r="B118" s="42"/>
       <c r="C118" s="8">
         <v>60</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E118" s="8"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B119" s="44"/>
+        <v>163</v>
+      </c>
+      <c r="B119" s="42"/>
       <c r="C119" s="8">
         <v>45</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E119" s="8"/>
     </row>
     <row r="120" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A120" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B120" s="42"/>
+      <c r="C120" s="8">
+        <v>60</v>
+      </c>
+      <c r="D120" s="9" t="s">
         <v>165</v>
-      </c>
-      <c r="B120" s="44"/>
-      <c r="C120" s="8">
-        <v>60</v>
-      </c>
-      <c r="D120" s="9" t="s">
-        <v>166</v>
       </c>
       <c r="E120" s="8"/>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="B121" s="44"/>
+        <v>166</v>
+      </c>
+      <c r="B121" s="42"/>
       <c r="C121" s="8">
         <v>35</v>
       </c>
       <c r="D121" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E121" s="8"/>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="B122" s="44"/>
+        <v>166</v>
+      </c>
+      <c r="B122" s="42"/>
       <c r="C122" s="8">
         <v>60</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E122" s="8"/>
     </row>
     <row r="123" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="B123" s="45"/>
+        <v>166</v>
+      </c>
+      <c r="B123" s="43"/>
       <c r="C123" s="8">
         <v>35</v>
       </c>
       <c r="D123" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E123" s="8"/>
     </row>
@@ -2927,114 +2972,114 @@
       <c r="A124" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B124" s="40" t="str">
+      <c r="B124" s="36" t="str">
         <f>INT(SUM(C114:C123)/60)&amp;"h"&amp;MOD(SUM(C114:C123),60)</f>
         <v>7h20</v>
       </c>
-      <c r="C124" s="41"/>
-      <c r="D124" s="41"/>
-      <c r="E124" s="42"/>
+      <c r="C124" s="37"/>
+      <c r="D124" s="37"/>
+      <c r="E124" s="38"/>
     </row>
     <row r="125" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A125" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="B125" s="43">
+        <v>171</v>
+      </c>
+      <c r="B125" s="41">
         <v>46163</v>
       </c>
       <c r="C125" s="13">
         <v>30</v>
       </c>
       <c r="D125" s="14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E125" s="13"/>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="B126" s="44"/>
+        <v>173</v>
+      </c>
+      <c r="B126" s="42"/>
       <c r="C126" s="8">
         <v>30</v>
       </c>
       <c r="D126" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E126" s="8"/>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B127" s="44"/>
+        <v>175</v>
+      </c>
+      <c r="B127" s="42"/>
       <c r="C127" s="8">
         <v>35</v>
       </c>
       <c r="D127" s="9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E127" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B128" s="44"/>
+        <v>175</v>
+      </c>
+      <c r="B128" s="42"/>
       <c r="C128" s="8">
         <v>60</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E128" s="8"/>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="B129" s="44"/>
+        <v>175</v>
+      </c>
+      <c r="B129" s="42"/>
       <c r="C129" s="8">
         <v>35</v>
       </c>
       <c r="D129" s="9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E129" s="8"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="8"/>
-      <c r="B130" s="44"/>
+      <c r="B130" s="42"/>
       <c r="C130" s="8"/>
       <c r="D130" s="9"/>
       <c r="E130" s="8"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="8"/>
-      <c r="B131" s="44"/>
+      <c r="B131" s="42"/>
       <c r="C131" s="8"/>
       <c r="D131" s="9"/>
       <c r="E131" s="8"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="8"/>
-      <c r="B132" s="44"/>
+      <c r="B132" s="42"/>
       <c r="C132" s="8"/>
       <c r="D132" s="9"/>
       <c r="E132" s="8"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="8"/>
-      <c r="B133" s="44"/>
+      <c r="B133" s="42"/>
       <c r="C133" s="8"/>
       <c r="D133" s="9"/>
       <c r="E133" s="8"/>
     </row>
     <row r="134" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8"/>
-      <c r="B134" s="45"/>
+      <c r="B134" s="43"/>
       <c r="C134" s="8"/>
       <c r="D134" s="9"/>
       <c r="E134" s="8"/>
@@ -3043,189 +3088,341 @@
       <c r="A135" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B135" s="40" t="str">
+      <c r="B135" s="36" t="str">
         <f>INT(SUM(C125:C134)/60)&amp;"h"&amp;MOD(SUM(C125:C134),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C135" s="41"/>
-      <c r="D135" s="41"/>
-      <c r="E135" s="42"/>
-    </row>
-    <row r="136" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="46" t="s">
+      <c r="C135" s="37"/>
+      <c r="D135" s="37"/>
+      <c r="E135" s="38"/>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="B136" s="41">
+        <v>46163</v>
+      </c>
+      <c r="C136" s="13">
+        <v>60</v>
+      </c>
+      <c r="D136" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="E136" s="13"/>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B137" s="42"/>
+      <c r="C137" s="8">
+        <v>35</v>
+      </c>
+      <c r="D137" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="E137" s="8"/>
+    </row>
+    <row r="138" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A138" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B138" s="42"/>
+      <c r="C138" s="8">
+        <v>60</v>
+      </c>
+      <c r="D138" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="E138" s="8"/>
+    </row>
+    <row r="139" spans="1:5" ht="81" x14ac:dyDescent="0.25">
+      <c r="A139" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B139" s="42"/>
+      <c r="C139" s="8">
+        <v>60</v>
+      </c>
+      <c r="D139" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E139" s="8"/>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B140" s="42"/>
+      <c r="C140" s="8">
+        <v>25</v>
+      </c>
+      <c r="D140" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="E140" s="8"/>
+    </row>
+    <row r="141" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A141" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B141" s="42"/>
+      <c r="C141" s="8">
+        <v>60</v>
+      </c>
+      <c r="D141" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="E141" s="8"/>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B142" s="42"/>
+      <c r="C142" s="8">
+        <v>40</v>
+      </c>
+      <c r="D142" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E142" s="8"/>
+    </row>
+    <row r="143" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A143" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="B143" s="42"/>
+      <c r="C143" s="8">
+        <v>60</v>
+      </c>
+      <c r="D143" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="E143" s="8"/>
+    </row>
+    <row r="144" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A144" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="B144" s="42"/>
+      <c r="C144" s="8">
+        <v>30</v>
+      </c>
+      <c r="D144" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="E144" s="8"/>
+    </row>
+    <row r="145" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="8"/>
+      <c r="B145" s="43"/>
+      <c r="C145" s="8"/>
+      <c r="D145" s="9"/>
+      <c r="E145" s="8"/>
+    </row>
+    <row r="146" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B146" s="36" t="str">
+        <f>INT(SUM(C136:C145)/60)&amp;"h"&amp;MOD(SUM(C136:C145),60)</f>
+        <v>7h10</v>
+      </c>
+      <c r="C146" s="37"/>
+      <c r="D146" s="37"/>
+      <c r="E146" s="38"/>
+    </row>
+    <row r="147" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A147" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B136" s="47"/>
-      <c r="C136" s="15">
-        <f>MROUND(SUM(C6:C135) /60,0.2)</f>
-        <v>74.400000000000006</v>
-      </c>
-      <c r="D136" s="16"/>
-      <c r="E136" s="17"/>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A138" s="18" t="s">
+      <c r="B147" s="40"/>
+      <c r="C147" s="15">
+        <f>MROUND(SUM(C6:C146) /60,0.2)</f>
+        <v>81.600000000000009</v>
+      </c>
+      <c r="D147" s="16"/>
+      <c r="E147" s="17"/>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A139" s="18"/>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C145" s="1" t="s">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" s="18"/>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E152" s="24"/>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E153" s="24"/>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E154" s="24"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E155" s="24"/>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C156" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D156" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="D145" s="35" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A147" s="1" t="s">
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C157" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D157" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E157" s="34"/>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C158" s="34">
+        <v>1.3555555555555556</v>
+      </c>
+      <c r="D158" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C147" s="34">
-        <v>1.1402777777777777</v>
-      </c>
-      <c r="D147" s="24">
-        <v>0.41666666666666669</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A149" s="1" t="s">
+      <c r="C160" s="24">
+        <v>6.5972222222222224E-2</v>
+      </c>
+      <c r="D160" s="24">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C149" s="24">
-        <v>6.5972222222222224E-2</v>
-      </c>
-      <c r="D149" s="24">
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A151" s="1" t="s">
+      <c r="C162" s="24">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D162" s="24">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E163" s="24"/>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C164" s="24">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="D164" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E164" s="24"/>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C151" s="24">
+      <c r="C166" s="24">
+        <v>0.15625</v>
+      </c>
+      <c r="D166" s="24">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C168" s="24">
+        <v>0.18402777777777779</v>
+      </c>
+      <c r="D168" s="24">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A170" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="C170" s="24">
+        <v>0.19791666666666666</v>
+      </c>
+      <c r="D170" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" ht="54" x14ac:dyDescent="0.25">
+      <c r="A172" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="C172" s="24">
+        <v>0.25347222222222221</v>
+      </c>
+      <c r="D172" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C174" s="24">
+        <v>0.11458333333333333</v>
+      </c>
+      <c r="D174" s="24">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C176" s="24">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="D151" s="24">
-        <v>0.125</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A153" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C153" s="24">
-        <v>0.1111111111111111</v>
-      </c>
-      <c r="D153" s="24">
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A155" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C155" s="24">
-        <v>0.11458333333333333</v>
-      </c>
-      <c r="D155" s="24">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A157" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="C157" s="24">
-        <v>0.15625</v>
-      </c>
-      <c r="D157" s="24">
-        <v>0.16666666666666666</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A159" s="33" t="s">
-        <v>153</v>
-      </c>
-      <c r="C159" s="24">
-        <v>0.19791666666666666</v>
-      </c>
-      <c r="D159" s="24">
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" ht="54" x14ac:dyDescent="0.25">
-      <c r="A161" s="33" t="s">
-        <v>154</v>
-      </c>
-      <c r="C161" s="24">
-        <v>0.13194444444444445</v>
-      </c>
-      <c r="D161" s="24">
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A163" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="C163" s="24">
-        <v>9.0277777777777776E-2</v>
-      </c>
-      <c r="D163" s="24">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A165" s="1" t="s">
+      <c r="D176" s="24">
+        <v>0.20833333333333334</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A178" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C178" s="34">
+        <f>C180 - SUM(C158:C176)</f>
+        <v>0.71388888888888857</v>
+      </c>
+      <c r="D178" s="48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C165" s="24">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D165" s="24">
-        <v>0.20833333333333334</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A167" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="C167" s="34">
-        <f>C169 - SUM(C147:C165)</f>
-        <v>0.57152777777777741</v>
-      </c>
-      <c r="D167" s="35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A169" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C169" s="34">
-        <v>2.7465277777777777</v>
+      <c r="C180" s="34">
+        <v>3.3194444444444446</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="33">
     <mergeCell ref="B135:E135"/>
-    <mergeCell ref="A136:B136"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B125:B134"/>
-    <mergeCell ref="B94:B102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B104:B112"/>
-    <mergeCell ref="B113:E113"/>
-    <mergeCell ref="B114:B123"/>
-    <mergeCell ref="B124:E124"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -3242,12 +3439,28 @@
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B55:B66"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="A147:B147"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B136:B145"/>
+    <mergeCell ref="B94:B102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B104:B112"/>
+    <mergeCell ref="B113:E113"/>
+    <mergeCell ref="B114:B123"/>
+    <mergeCell ref="B124:E124"/>
+    <mergeCell ref="B125:B134"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C125:C134 C19:C27 C94:C102 C104:C112 C114:C123" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C136:C145 C19:C27 C94:C102 C104:C112 C114:C123 C125:C134" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B125:B134 B94:B102 B104:B112 B114:B123" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B136:B145 B94:B102 B104:B112 B114:B123 B125:B134" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -3256,7 +3469,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="25" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="23" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -3426,11 +3639,14 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E16" s="26"/>
     </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E19" s="26"/>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
       <c r="E20" s="26"/>
+    </row>
+    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C22" s="26"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D33" s="26"/>
@@ -3448,6 +3664,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -3609,15 +3834,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -3635,6 +3851,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3650,12 +3874,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update(NL): change delete system
</commit_message>
<xml_diff>
--- a/Doc/ThomNardou-JDT.xlsx
+++ b/Doc/ThomNardou-JDT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk88yte\Documents\Github\Agora\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03587A42-8D40-417D-9C43-2AA5CC47256F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82CE9C36-9B69-47C2-8857-2C8CE6DB4D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Feuil1" sheetId="19" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$147</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$158</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="197">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -635,6 +635,15 @@
   </si>
   <si>
     <t>J'ai commencé à modifier le système de suppression</t>
+  </si>
+  <si>
+    <t>J'ai modififé la vidéo j'ai réussi à ce qu'elle fasse 41sec mais je vais arreter de toucher plus car sinon ca va pas être lisible</t>
+  </si>
+  <si>
+    <t>Système de supression</t>
+  </si>
+  <si>
+    <t>J'ai modifié le système de suppression"miantenant une campagne et juste en annulée si elle est planifiée à la base</t>
   </si>
 </sst>
 </file>
@@ -998,6 +1007,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -1010,11 +1022,17 @@
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1028,20 +1046,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1359,7 +1368,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G180"/>
+  <dimension ref="A1:G191"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" style="1" customWidth="1"/>
@@ -1375,10 +1384,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="44"/>
+      <c r="C1" s="40"/>
       <c r="D1" s="22" t="s">
         <v>1</v>
       </c>
@@ -1390,10 +1399,10 @@
       <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="44"/>
+      <c r="C2" s="40"/>
       <c r="D2" s="22" t="s">
         <v>3</v>
       </c>
@@ -1405,10 +1414,10 @@
       <c r="A3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="44"/>
+      <c r="C3" s="40"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
@@ -1420,12 +1429,12 @@
       <c r="A4" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="47"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1448,7 +1457,7 @@
       <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="41">
+      <c r="B6" s="44">
         <v>46139</v>
       </c>
       <c r="C6" s="5">
@@ -1461,7 +1470,7 @@
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="42"/>
+      <c r="B7" s="45"/>
       <c r="C7" s="8">
         <v>30</v>
       </c>
@@ -1474,7 +1483,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="42"/>
+      <c r="B8" s="45"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
@@ -1487,7 +1496,7 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="42"/>
+      <c r="B9" s="45"/>
       <c r="C9" s="8">
         <v>10</v>
       </c>
@@ -1498,7 +1507,7 @@
       <c r="A10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="42"/>
+      <c r="B10" s="45"/>
       <c r="C10" s="10">
         <v>20</v>
       </c>
@@ -1511,7 +1520,7 @@
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="42"/>
+      <c r="B11" s="45"/>
       <c r="C11" s="10">
         <v>20</v>
       </c>
@@ -1526,7 +1535,7 @@
       <c r="A12" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="42"/>
+      <c r="B12" s="45"/>
       <c r="C12" s="10">
         <v>60</v>
       </c>
@@ -1541,7 +1550,7 @@
       <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="42"/>
+      <c r="B13" s="45"/>
       <c r="C13" s="10">
         <v>10</v>
       </c>
@@ -1556,7 +1565,7 @@
       <c r="A14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="42"/>
+      <c r="B14" s="45"/>
       <c r="C14" s="10">
         <v>60</v>
       </c>
@@ -1571,7 +1580,7 @@
       <c r="A15" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="42"/>
+      <c r="B15" s="45"/>
       <c r="C15" s="10">
         <v>45</v>
       </c>
@@ -1586,7 +1595,7 @@
       <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="42"/>
+      <c r="B16" s="45"/>
       <c r="C16" s="10">
         <v>20</v>
       </c>
@@ -1599,7 +1608,7 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7"/>
-      <c r="B17" s="43"/>
+      <c r="B17" s="46"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1608,19 +1617,19 @@
       <c r="A18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="36" t="str">
+      <c r="B18" s="37" t="str">
         <f>INT(SUM(C6:C17)/60)&amp;"h"&amp;MOD(SUM(C6:C17),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="39"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="41">
+      <c r="B19" s="44">
         <v>46141</v>
       </c>
       <c r="C19" s="5">
@@ -1635,7 +1644,7 @@
       <c r="A20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="42"/>
+      <c r="B20" s="45"/>
       <c r="C20" s="8">
         <v>55</v>
       </c>
@@ -1648,7 +1657,7 @@
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B21" s="42"/>
+      <c r="B21" s="45"/>
       <c r="C21" s="8">
         <v>40</v>
       </c>
@@ -1662,7 +1671,7 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="42"/>
+      <c r="B22" s="45"/>
       <c r="C22" s="8">
         <v>45</v>
       </c>
@@ -1675,7 +1684,7 @@
       <c r="A23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="42"/>
+      <c r="B23" s="45"/>
       <c r="C23" s="10">
         <v>60</v>
       </c>
@@ -1688,7 +1697,7 @@
       <c r="A24" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="42"/>
+      <c r="B24" s="45"/>
       <c r="C24" s="10">
         <v>60</v>
       </c>
@@ -1701,7 +1710,7 @@
       <c r="A25" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="42"/>
+      <c r="B25" s="45"/>
       <c r="C25" s="10">
         <v>30</v>
       </c>
@@ -1714,7 +1723,7 @@
       <c r="A26" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="42"/>
+      <c r="B26" s="45"/>
       <c r="C26" s="10">
         <v>60</v>
       </c>
@@ -1727,7 +1736,7 @@
       <c r="A27" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="43"/>
+      <c r="B27" s="46"/>
       <c r="C27" s="10">
         <v>40</v>
       </c>
@@ -1740,19 +1749,19 @@
       <c r="A28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="36" t="str">
+      <c r="B28" s="37" t="str">
         <f>INT(SUM(C19:C27)/60)&amp;"h"&amp;MOD(SUM(C19:C27),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C28" s="37"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="39"/>
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="41">
+      <c r="B29" s="44">
         <v>46142</v>
       </c>
       <c r="C29" s="5">
@@ -1767,7 +1776,7 @@
       <c r="A30" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="42"/>
+      <c r="B30" s="45"/>
       <c r="C30" s="8">
         <v>60</v>
       </c>
@@ -1782,7 +1791,7 @@
       <c r="A31" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="42"/>
+      <c r="B31" s="45"/>
       <c r="C31" s="8">
         <v>70</v>
       </c>
@@ -1793,14 +1802,14 @@
     </row>
     <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
-      <c r="B32" s="42"/>
+      <c r="B32" s="45"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="10"/>
-      <c r="B33" s="43"/>
+      <c r="B33" s="46"/>
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="10"/>
@@ -1809,19 +1818,19 @@
       <c r="A34" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="36" t="str">
+      <c r="B34" s="37" t="str">
         <f>INT(SUM(C29:C33)/60)&amp;"h"&amp;MOD(SUM(C29:C33),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C34" s="37"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="39"/>
     </row>
     <row r="35" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B35" s="41">
+      <c r="B35" s="44">
         <v>46143</v>
       </c>
       <c r="C35" s="5">
@@ -1836,7 +1845,7 @@
       <c r="A36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="42"/>
+      <c r="B36" s="45"/>
       <c r="C36" s="8">
         <v>35</v>
       </c>
@@ -1849,7 +1858,7 @@
       <c r="A37" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="42"/>
+      <c r="B37" s="45"/>
       <c r="C37" s="8">
         <v>60</v>
       </c>
@@ -1862,7 +1871,7 @@
       <c r="A38" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B38" s="42"/>
+      <c r="B38" s="45"/>
       <c r="C38" s="8">
         <v>30</v>
       </c>
@@ -1875,7 +1884,7 @@
       <c r="A39" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="B39" s="42"/>
+      <c r="B39" s="45"/>
       <c r="C39" s="10">
         <v>35</v>
       </c>
@@ -1888,7 +1897,7 @@
       <c r="A40" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B40" s="42"/>
+      <c r="B40" s="45"/>
       <c r="C40" s="10">
         <v>20</v>
       </c>
@@ -1901,7 +1910,7 @@
       <c r="A41" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B41" s="42"/>
+      <c r="B41" s="45"/>
       <c r="C41" s="10">
         <v>50</v>
       </c>
@@ -1914,7 +1923,7 @@
       <c r="A42" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B42" s="42"/>
+      <c r="B42" s="45"/>
       <c r="C42" s="10">
         <v>45</v>
       </c>
@@ -1927,7 +1936,7 @@
       <c r="A43" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B43" s="42"/>
+      <c r="B43" s="45"/>
       <c r="C43" s="10">
         <v>60</v>
       </c>
@@ -1940,7 +1949,7 @@
       <c r="A44" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B44" s="43"/>
+      <c r="B44" s="46"/>
       <c r="C44" s="10">
         <v>35</v>
       </c>
@@ -1953,19 +1962,19 @@
       <c r="A45" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="36" t="str">
+      <c r="B45" s="37" t="str">
         <f>INT(SUM(C35:C44)/60)&amp;"h"&amp;MOD(SUM(C35:C44),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C45" s="37"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="39"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="B46" s="41">
+      <c r="B46" s="44">
         <v>46146</v>
       </c>
       <c r="C46" s="13">
@@ -1980,7 +1989,7 @@
       <c r="A47" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B47" s="42"/>
+      <c r="B47" s="45"/>
       <c r="C47" s="8">
         <v>45</v>
       </c>
@@ -1993,7 +2002,7 @@
       <c r="A48" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B48" s="42"/>
+      <c r="B48" s="45"/>
       <c r="C48" s="8">
         <v>60</v>
       </c>
@@ -2006,7 +2015,7 @@
       <c r="A49" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="42"/>
+      <c r="B49" s="45"/>
       <c r="C49" s="8">
         <v>35</v>
       </c>
@@ -2019,7 +2028,7 @@
       <c r="A50" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B50" s="42"/>
+      <c r="B50" s="45"/>
       <c r="C50" s="8">
         <v>60</v>
       </c>
@@ -2032,7 +2041,7 @@
       <c r="A51" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="B51" s="42"/>
+      <c r="B51" s="45"/>
       <c r="C51" s="8">
         <v>20</v>
       </c>
@@ -2045,7 +2054,7 @@
       <c r="A52" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B52" s="42"/>
+      <c r="B52" s="45"/>
       <c r="C52" s="8">
         <v>55</v>
       </c>
@@ -2056,7 +2065,7 @@
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="8"/>
-      <c r="B53" s="43"/>
+      <c r="B53" s="46"/>
       <c r="C53" s="8"/>
       <c r="D53" s="32"/>
       <c r="E53" s="31"/>
@@ -2065,19 +2074,19 @@
       <c r="A54" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B54" s="36" t="str">
+      <c r="B54" s="37" t="str">
         <f>INT(SUM(C46:C53)/60)&amp;"h"&amp;MOD(SUM(C46:C53),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C54" s="37"/>
-      <c r="D54" s="37"/>
-      <c r="E54" s="38"/>
+      <c r="C54" s="38"/>
+      <c r="D54" s="38"/>
+      <c r="E54" s="39"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B55" s="41">
+      <c r="B55" s="44">
         <v>46148</v>
       </c>
       <c r="C55" s="5">
@@ -2092,7 +2101,7 @@
       <c r="A56" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B56" s="42"/>
+      <c r="B56" s="45"/>
       <c r="C56" s="8">
         <v>35</v>
       </c>
@@ -2105,7 +2114,7 @@
       <c r="A57" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B57" s="42"/>
+      <c r="B57" s="45"/>
       <c r="C57" s="8">
         <v>60</v>
       </c>
@@ -2118,7 +2127,7 @@
       <c r="A58" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B58" s="42"/>
+      <c r="B58" s="45"/>
       <c r="C58" s="8">
         <v>60</v>
       </c>
@@ -2131,7 +2140,7 @@
       <c r="A59" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="B59" s="42"/>
+      <c r="B59" s="45"/>
       <c r="C59" s="10">
         <v>40</v>
       </c>
@@ -2144,7 +2153,7 @@
       <c r="A60" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="B60" s="42"/>
+      <c r="B60" s="45"/>
       <c r="C60" s="10">
         <v>10</v>
       </c>
@@ -2157,7 +2166,7 @@
       <c r="A61" s="28" t="s">
         <v>97</v>
       </c>
-      <c r="B61" s="42"/>
+      <c r="B61" s="45"/>
       <c r="C61" s="10">
         <v>20</v>
       </c>
@@ -2170,7 +2179,7 @@
       <c r="A62" s="28" t="s">
         <v>94</v>
       </c>
-      <c r="B62" s="42"/>
+      <c r="B62" s="45"/>
       <c r="C62" s="10">
         <v>20</v>
       </c>
@@ -2183,7 +2192,7 @@
       <c r="A63" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="B63" s="42"/>
+      <c r="B63" s="45"/>
       <c r="C63" s="10">
         <v>35</v>
       </c>
@@ -2198,7 +2207,7 @@
       <c r="A64" s="28" t="s">
         <v>187</v>
       </c>
-      <c r="B64" s="42"/>
+      <c r="B64" s="45"/>
       <c r="C64" s="10">
         <v>45</v>
       </c>
@@ -2211,7 +2220,7 @@
       <c r="A65" s="28" t="s">
         <v>187</v>
       </c>
-      <c r="B65" s="42"/>
+      <c r="B65" s="45"/>
       <c r="C65" s="10">
         <v>45</v>
       </c>
@@ -2222,7 +2231,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="43"/>
+      <c r="B66" s="46"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -2231,19 +2240,19 @@
       <c r="A67" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B67" s="36" t="str">
+      <c r="B67" s="37" t="str">
         <f>INT(SUM(C55:C66)/60)&amp;"h"&amp;MOD(SUM(C55:C66),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C67" s="37"/>
-      <c r="D67" s="37"/>
-      <c r="E67" s="38"/>
+      <c r="C67" s="38"/>
+      <c r="D67" s="38"/>
+      <c r="E67" s="39"/>
     </row>
     <row r="68" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B68" s="41">
+      <c r="B68" s="44">
         <v>46149</v>
       </c>
       <c r="C68" s="5">
@@ -2258,7 +2267,7 @@
       <c r="A69" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B69" s="42"/>
+      <c r="B69" s="45"/>
       <c r="C69" s="8">
         <v>60</v>
       </c>
@@ -2271,7 +2280,7 @@
       <c r="A70" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B70" s="42"/>
+      <c r="B70" s="45"/>
       <c r="C70" s="8">
         <v>55</v>
       </c>
@@ -2284,7 +2293,7 @@
       <c r="A71" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B71" s="42"/>
+      <c r="B71" s="45"/>
       <c r="C71" s="8">
         <v>15</v>
       </c>
@@ -2295,7 +2304,7 @@
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="10"/>
-      <c r="B72" s="43"/>
+      <c r="B72" s="46"/>
       <c r="C72" s="10"/>
       <c r="D72" s="11"/>
       <c r="E72" s="10"/>
@@ -2304,19 +2313,19 @@
       <c r="A73" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B73" s="36" t="str">
+      <c r="B73" s="37" t="str">
         <f>INT(SUM(C68:C72)/60)&amp;"h"&amp;MOD(SUM(C68:C72),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C73" s="37"/>
-      <c r="D73" s="37"/>
-      <c r="E73" s="38"/>
+      <c r="C73" s="38"/>
+      <c r="D73" s="38"/>
+      <c r="E73" s="39"/>
     </row>
     <row r="74" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B74" s="41">
+      <c r="B74" s="44">
         <v>46150</v>
       </c>
       <c r="C74" s="5">
@@ -2331,7 +2340,7 @@
       <c r="A75" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="42"/>
+      <c r="B75" s="45"/>
       <c r="C75" s="8">
         <v>50</v>
       </c>
@@ -2344,7 +2353,7 @@
       <c r="A76" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B76" s="42"/>
+      <c r="B76" s="45"/>
       <c r="C76" s="8">
         <v>35</v>
       </c>
@@ -2357,7 +2366,7 @@
       <c r="A77" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B77" s="42"/>
+      <c r="B77" s="45"/>
       <c r="C77" s="8">
         <v>60</v>
       </c>
@@ -2370,7 +2379,7 @@
       <c r="A78" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="B78" s="42"/>
+      <c r="B78" s="45"/>
       <c r="C78" s="10">
         <v>60</v>
       </c>
@@ -2383,7 +2392,7 @@
       <c r="A79" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B79" s="42"/>
+      <c r="B79" s="45"/>
       <c r="C79" s="10">
         <v>25</v>
       </c>
@@ -2396,7 +2405,7 @@
       <c r="A80" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B80" s="42"/>
+      <c r="B80" s="45"/>
       <c r="C80" s="10">
         <v>60</v>
       </c>
@@ -2409,7 +2418,7 @@
       <c r="A81" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B81" s="42"/>
+      <c r="B81" s="45"/>
       <c r="C81" s="10">
         <v>60</v>
       </c>
@@ -2422,7 +2431,7 @@
       <c r="A82" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B82" s="42"/>
+      <c r="B82" s="45"/>
       <c r="C82" s="10">
         <v>60</v>
       </c>
@@ -2435,7 +2444,7 @@
       <c r="A83" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B83" s="43"/>
+      <c r="B83" s="46"/>
       <c r="C83" s="10">
         <v>10</v>
       </c>
@@ -2448,19 +2457,19 @@
       <c r="A84" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B84" s="36" t="str">
+      <c r="B84" s="37" t="str">
         <f>INT(SUM(C74:C83)/60)&amp;"h"&amp;MOD(SUM(C74:C83),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C84" s="37"/>
-      <c r="D84" s="37"/>
-      <c r="E84" s="38"/>
+      <c r="C84" s="38"/>
+      <c r="D84" s="38"/>
+      <c r="E84" s="39"/>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="41">
+      <c r="B85" s="44">
         <v>46153</v>
       </c>
       <c r="C85" s="5">
@@ -2475,7 +2484,7 @@
       <c r="A86" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="B86" s="42"/>
+      <c r="B86" s="45"/>
       <c r="C86" s="8">
         <v>40</v>
       </c>
@@ -2488,7 +2497,7 @@
       <c r="A87" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B87" s="42"/>
+      <c r="B87" s="45"/>
       <c r="C87" s="8">
         <v>60</v>
       </c>
@@ -2501,7 +2510,7 @@
       <c r="A88" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B88" s="42"/>
+      <c r="B88" s="45"/>
       <c r="C88" s="8">
         <v>60</v>
       </c>
@@ -2514,7 +2523,7 @@
       <c r="A89" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B89" s="42"/>
+      <c r="B89" s="45"/>
       <c r="C89" s="10">
         <v>15</v>
       </c>
@@ -2527,7 +2536,7 @@
       <c r="A90" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B90" s="42"/>
+      <c r="B90" s="45"/>
       <c r="C90" s="10">
         <v>60</v>
       </c>
@@ -2540,7 +2549,7 @@
       <c r="A91" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B91" s="42"/>
+      <c r="B91" s="45"/>
       <c r="C91" s="10">
         <v>60</v>
       </c>
@@ -2553,7 +2562,7 @@
       <c r="A92" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B92" s="43"/>
+      <c r="B92" s="46"/>
       <c r="C92" s="10">
         <v>10</v>
       </c>
@@ -2566,19 +2575,19 @@
       <c r="A93" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B93" s="36" t="str">
+      <c r="B93" s="37" t="str">
         <f>INT(SUM(C85:C92)/60)&amp;"h"&amp;MOD(SUM(C85:C92),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C93" s="37"/>
-      <c r="D93" s="37"/>
-      <c r="E93" s="38"/>
+      <c r="C93" s="38"/>
+      <c r="D93" s="38"/>
+      <c r="E93" s="39"/>
     </row>
     <row r="94" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B94" s="41">
+      <c r="B94" s="44">
         <v>46155</v>
       </c>
       <c r="C94" s="13">
@@ -2593,7 +2602,7 @@
       <c r="A95" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B95" s="42"/>
+      <c r="B95" s="45"/>
       <c r="C95" s="8">
         <v>35</v>
       </c>
@@ -2606,7 +2615,7 @@
       <c r="A96" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B96" s="42"/>
+      <c r="B96" s="45"/>
       <c r="C96" s="8">
         <v>60</v>
       </c>
@@ -2619,7 +2628,7 @@
       <c r="A97" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B97" s="42"/>
+      <c r="B97" s="45"/>
       <c r="C97" s="8">
         <v>60</v>
       </c>
@@ -2632,7 +2641,7 @@
       <c r="A98" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B98" s="42"/>
+      <c r="B98" s="45"/>
       <c r="C98" s="8">
         <v>25</v>
       </c>
@@ -2645,7 +2654,7 @@
       <c r="A99" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B99" s="42"/>
+      <c r="B99" s="45"/>
       <c r="C99" s="8">
         <v>60</v>
       </c>
@@ -2658,7 +2667,7 @@
       <c r="A100" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B100" s="42"/>
+      <c r="B100" s="45"/>
       <c r="C100" s="8">
         <v>45</v>
       </c>
@@ -2671,7 +2680,7 @@
       <c r="A101" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B101" s="42"/>
+      <c r="B101" s="45"/>
       <c r="C101" s="8">
         <v>60</v>
       </c>
@@ -2684,7 +2693,7 @@
       <c r="A102" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B102" s="43"/>
+      <c r="B102" s="46"/>
       <c r="C102" s="8">
         <v>25</v>
       </c>
@@ -2697,19 +2706,19 @@
       <c r="A103" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B103" s="36" t="str">
+      <c r="B103" s="37" t="str">
         <f>INT(SUM(C94:C102)/60)&amp;"h"&amp;MOD(SUM(C94:C102),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C103" s="37"/>
-      <c r="D103" s="37"/>
-      <c r="E103" s="38"/>
+      <c r="C103" s="38"/>
+      <c r="D103" s="38"/>
+      <c r="E103" s="39"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="B104" s="41">
+      <c r="B104" s="44">
         <v>46160</v>
       </c>
       <c r="C104" s="13">
@@ -2724,7 +2733,7 @@
       <c r="A105" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B105" s="42"/>
+      <c r="B105" s="45"/>
       <c r="C105" s="8">
         <v>22</v>
       </c>
@@ -2737,7 +2746,7 @@
       <c r="A106" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B106" s="42"/>
+      <c r="B106" s="45"/>
       <c r="C106" s="8">
         <v>20</v>
       </c>
@@ -2750,7 +2759,7 @@
       <c r="A107" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B107" s="42"/>
+      <c r="B107" s="45"/>
       <c r="C107" s="8">
         <v>25</v>
       </c>
@@ -2763,7 +2772,7 @@
       <c r="A108" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B108" s="42"/>
+      <c r="B108" s="45"/>
       <c r="C108" s="8">
         <v>40</v>
       </c>
@@ -2776,7 +2785,7 @@
       <c r="A109" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B109" s="42"/>
+      <c r="B109" s="45"/>
       <c r="C109" s="8">
         <v>55</v>
       </c>
@@ -2789,7 +2798,7 @@
       <c r="A110" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B110" s="42"/>
+      <c r="B110" s="45"/>
       <c r="C110" s="8">
         <v>60</v>
       </c>
@@ -2802,7 +2811,7 @@
       <c r="A111" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B111" s="42"/>
+      <c r="B111" s="45"/>
       <c r="C111" s="8">
         <v>60</v>
       </c>
@@ -2815,7 +2824,7 @@
       <c r="A112" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B112" s="43"/>
+      <c r="B112" s="46"/>
       <c r="C112" s="8">
         <v>15</v>
       </c>
@@ -2828,19 +2837,19 @@
       <c r="A113" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B113" s="36" t="str">
+      <c r="B113" s="37" t="str">
         <f>INT(SUM(C104:C112)/60)&amp;"h"&amp;MOD(SUM(C104:C112),60)</f>
         <v>5h25</v>
       </c>
-      <c r="C113" s="37"/>
-      <c r="D113" s="37"/>
-      <c r="E113" s="38"/>
+      <c r="C113" s="38"/>
+      <c r="D113" s="38"/>
+      <c r="E113" s="39"/>
     </row>
     <row r="114" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A114" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B114" s="41">
+      <c r="B114" s="44">
         <v>46162</v>
       </c>
       <c r="C114" s="13">
@@ -2855,7 +2864,7 @@
       <c r="A115" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B115" s="42"/>
+      <c r="B115" s="45"/>
       <c r="C115" s="8">
         <v>35</v>
       </c>
@@ -2868,7 +2877,7 @@
       <c r="A116" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B116" s="42"/>
+      <c r="B116" s="45"/>
       <c r="C116" s="8">
         <v>20</v>
       </c>
@@ -2881,7 +2890,7 @@
       <c r="A117" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="B117" s="42"/>
+      <c r="B117" s="45"/>
       <c r="C117" s="8">
         <v>30</v>
       </c>
@@ -2894,7 +2903,7 @@
       <c r="A118" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="B118" s="42"/>
+      <c r="B118" s="45"/>
       <c r="C118" s="8">
         <v>60</v>
       </c>
@@ -2907,7 +2916,7 @@
       <c r="A119" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="B119" s="42"/>
+      <c r="B119" s="45"/>
       <c r="C119" s="8">
         <v>45</v>
       </c>
@@ -2920,7 +2929,7 @@
       <c r="A120" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="B120" s="42"/>
+      <c r="B120" s="45"/>
       <c r="C120" s="8">
         <v>60</v>
       </c>
@@ -2933,7 +2942,7 @@
       <c r="A121" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B121" s="42"/>
+      <c r="B121" s="45"/>
       <c r="C121" s="8">
         <v>35</v>
       </c>
@@ -2946,7 +2955,7 @@
       <c r="A122" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B122" s="42"/>
+      <c r="B122" s="45"/>
       <c r="C122" s="8">
         <v>60</v>
       </c>
@@ -2959,7 +2968,7 @@
       <c r="A123" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="B123" s="43"/>
+      <c r="B123" s="46"/>
       <c r="C123" s="8">
         <v>35</v>
       </c>
@@ -2972,19 +2981,19 @@
       <c r="A124" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B124" s="36" t="str">
+      <c r="B124" s="37" t="str">
         <f>INT(SUM(C114:C123)/60)&amp;"h"&amp;MOD(SUM(C114:C123),60)</f>
         <v>7h20</v>
       </c>
-      <c r="C124" s="37"/>
-      <c r="D124" s="37"/>
-      <c r="E124" s="38"/>
+      <c r="C124" s="38"/>
+      <c r="D124" s="38"/>
+      <c r="E124" s="39"/>
     </row>
     <row r="125" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A125" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="B125" s="41">
+      <c r="B125" s="44">
         <v>46163</v>
       </c>
       <c r="C125" s="13">
@@ -2999,7 +3008,7 @@
       <c r="A126" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="B126" s="42"/>
+      <c r="B126" s="45"/>
       <c r="C126" s="8">
         <v>30</v>
       </c>
@@ -3012,7 +3021,7 @@
       <c r="A127" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="B127" s="42"/>
+      <c r="B127" s="45"/>
       <c r="C127" s="8">
         <v>35</v>
       </c>
@@ -3027,7 +3036,7 @@
       <c r="A128" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="B128" s="42"/>
+      <c r="B128" s="45"/>
       <c r="C128" s="8">
         <v>60</v>
       </c>
@@ -3040,7 +3049,7 @@
       <c r="A129" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="B129" s="42"/>
+      <c r="B129" s="45"/>
       <c r="C129" s="8">
         <v>35</v>
       </c>
@@ -3051,35 +3060,35 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="8"/>
-      <c r="B130" s="42"/>
+      <c r="B130" s="45"/>
       <c r="C130" s="8"/>
       <c r="D130" s="9"/>
       <c r="E130" s="8"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="8"/>
-      <c r="B131" s="42"/>
+      <c r="B131" s="45"/>
       <c r="C131" s="8"/>
       <c r="D131" s="9"/>
       <c r="E131" s="8"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="8"/>
-      <c r="B132" s="42"/>
+      <c r="B132" s="45"/>
       <c r="C132" s="8"/>
       <c r="D132" s="9"/>
       <c r="E132" s="8"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="8"/>
-      <c r="B133" s="42"/>
+      <c r="B133" s="45"/>
       <c r="C133" s="8"/>
       <c r="D133" s="9"/>
       <c r="E133" s="8"/>
     </row>
     <row r="134" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8"/>
-      <c r="B134" s="43"/>
+      <c r="B134" s="46"/>
       <c r="C134" s="8"/>
       <c r="D134" s="9"/>
       <c r="E134" s="8"/>
@@ -3088,20 +3097,20 @@
       <c r="A135" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B135" s="36" t="str">
+      <c r="B135" s="37" t="str">
         <f>INT(SUM(C125:C134)/60)&amp;"h"&amp;MOD(SUM(C125:C134),60)</f>
         <v>3h10</v>
       </c>
-      <c r="C135" s="37"/>
-      <c r="D135" s="37"/>
-      <c r="E135" s="38"/>
+      <c r="C135" s="38"/>
+      <c r="D135" s="38"/>
+      <c r="E135" s="39"/>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="B136" s="41">
-        <v>46163</v>
+      <c r="B136" s="44">
+        <v>46164</v>
       </c>
       <c r="C136" s="13">
         <v>60</v>
@@ -3115,7 +3124,7 @@
       <c r="A137" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="B137" s="42"/>
+      <c r="B137" s="45"/>
       <c r="C137" s="8">
         <v>35</v>
       </c>
@@ -3128,7 +3137,7 @@
       <c r="A138" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="B138" s="42"/>
+      <c r="B138" s="45"/>
       <c r="C138" s="8">
         <v>60</v>
       </c>
@@ -3141,7 +3150,7 @@
       <c r="A139" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="B139" s="42"/>
+      <c r="B139" s="45"/>
       <c r="C139" s="8">
         <v>60</v>
       </c>
@@ -3154,7 +3163,7 @@
       <c r="A140" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="B140" s="42"/>
+      <c r="B140" s="45"/>
       <c r="C140" s="8">
         <v>25</v>
       </c>
@@ -3167,7 +3176,7 @@
       <c r="A141" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="B141" s="42"/>
+      <c r="B141" s="45"/>
       <c r="C141" s="8">
         <v>60</v>
       </c>
@@ -3180,7 +3189,7 @@
       <c r="A142" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B142" s="42"/>
+      <c r="B142" s="45"/>
       <c r="C142" s="8">
         <v>40</v>
       </c>
@@ -3193,7 +3202,7 @@
       <c r="A143" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="B143" s="42"/>
+      <c r="B143" s="45"/>
       <c r="C143" s="8">
         <v>60</v>
       </c>
@@ -3206,7 +3215,7 @@
       <c r="A144" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="B144" s="42"/>
+      <c r="B144" s="45"/>
       <c r="C144" s="8">
         <v>30</v>
       </c>
@@ -3217,7 +3226,7 @@
     </row>
     <row r="145" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="8"/>
-      <c r="B145" s="43"/>
+      <c r="B145" s="46"/>
       <c r="C145" s="8"/>
       <c r="D145" s="9"/>
       <c r="E145" s="8"/>
@@ -3226,202 +3235,317 @@
       <c r="A146" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B146" s="36" t="str">
+      <c r="B146" s="37" t="str">
         <f>INT(SUM(C136:C145)/60)&amp;"h"&amp;MOD(SUM(C136:C145),60)</f>
         <v>7h10</v>
       </c>
-      <c r="C146" s="37"/>
-      <c r="D146" s="37"/>
-      <c r="E146" s="38"/>
-    </row>
-    <row r="147" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A147" s="39" t="s">
+      <c r="C146" s="38"/>
+      <c r="D146" s="38"/>
+      <c r="E146" s="39"/>
+    </row>
+    <row r="147" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A147" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B147" s="44">
+        <v>46169</v>
+      </c>
+      <c r="C147" s="13">
+        <v>20</v>
+      </c>
+      <c r="D147" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="E147" s="13"/>
+    </row>
+    <row r="148" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A148" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B148" s="45"/>
+      <c r="C148" s="8">
+        <v>20</v>
+      </c>
+      <c r="D148" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="E148" s="8"/>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" s="8"/>
+      <c r="B149" s="45"/>
+      <c r="C149" s="8"/>
+      <c r="D149" s="9"/>
+      <c r="E149" s="8"/>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" s="8"/>
+      <c r="B150" s="45"/>
+      <c r="C150" s="8"/>
+      <c r="D150" s="9"/>
+      <c r="E150" s="8"/>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" s="8"/>
+      <c r="B151" s="45"/>
+      <c r="C151" s="8"/>
+      <c r="D151" s="9"/>
+      <c r="E151" s="8"/>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" s="8"/>
+      <c r="B152" s="45"/>
+      <c r="C152" s="8"/>
+      <c r="D152" s="9"/>
+      <c r="E152" s="8"/>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" s="8"/>
+      <c r="B153" s="45"/>
+      <c r="C153" s="8"/>
+      <c r="D153" s="9"/>
+      <c r="E153" s="8"/>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" s="8"/>
+      <c r="B154" s="45"/>
+      <c r="C154" s="8"/>
+      <c r="D154" s="9"/>
+      <c r="E154" s="8"/>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" s="8"/>
+      <c r="B155" s="45"/>
+      <c r="C155" s="8"/>
+      <c r="D155" s="9"/>
+      <c r="E155" s="8"/>
+    </row>
+    <row r="156" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="8"/>
+      <c r="B156" s="46"/>
+      <c r="C156" s="8"/>
+      <c r="D156" s="9"/>
+      <c r="E156" s="8"/>
+    </row>
+    <row r="157" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B157" s="37" t="str">
+        <f>INT(SUM(C147:C156)/60)&amp;"h"&amp;MOD(SUM(C147:C156),60)</f>
+        <v>0h40</v>
+      </c>
+      <c r="C157" s="38"/>
+      <c r="D157" s="38"/>
+      <c r="E157" s="39"/>
+    </row>
+    <row r="158" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A158" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="B147" s="40"/>
-      <c r="C147" s="15">
-        <f>MROUND(SUM(C6:C146) /60,0.2)</f>
-        <v>81.600000000000009</v>
-      </c>
-      <c r="D147" s="16"/>
-      <c r="E147" s="17"/>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A149" s="18" t="s">
+      <c r="B158" s="48"/>
+      <c r="C158" s="15">
+        <f>MROUND(SUM(C6:C157) /60,0.2)</f>
+        <v>82.2</v>
+      </c>
+      <c r="D158" s="16"/>
+      <c r="E158" s="17"/>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A150" s="18"/>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E152" s="24"/>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E153" s="24"/>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E154" s="24"/>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E155" s="24"/>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C156" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="D156" s="35" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A157" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="C157" s="24">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="D157" s="24">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E157" s="34"/>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A158" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C158" s="34">
-        <v>1.3555555555555556</v>
-      </c>
-      <c r="D158" s="24">
-        <v>0.41666666666666669</v>
-      </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A160" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="C160" s="24">
-        <v>6.5972222222222224E-2</v>
-      </c>
-      <c r="D160" s="24">
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A162" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C162" s="24">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D162" s="24">
-        <v>0.125</v>
-      </c>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" s="18"/>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E163" s="24"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A164" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C164" s="24">
-        <v>0.1111111111111111</v>
-      </c>
-      <c r="D164" s="24">
-        <v>0.33333333333333331</v>
-      </c>
       <c r="E164" s="24"/>
     </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E165" s="24"/>
+    </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A166" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="C166" s="24">
-        <v>0.15625</v>
-      </c>
-      <c r="D166" s="24">
-        <v>0.25</v>
+      <c r="E166" s="24"/>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C167" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D167" s="35" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C168" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D168" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E168" s="34"/>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C169" s="34">
+        <v>1.3555555555555556</v>
+      </c>
+      <c r="D169" s="24">
+        <v>0.41666666666666669</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C171" s="24">
+        <v>6.5972222222222224E-2</v>
+      </c>
+      <c r="D171" s="24">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C173" s="24">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D173" s="24">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E174" s="24"/>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C175" s="24">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="D175" s="24">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="E175" s="24"/>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A177" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C177" s="24">
+        <v>0.15625</v>
+      </c>
+      <c r="D177" s="24">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A179" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C168" s="24">
+      <c r="C179" s="24">
         <v>0.18402777777777779</v>
       </c>
-      <c r="D168" s="24">
+      <c r="D179" s="24">
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="170" spans="1:5" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A170" s="33" t="s">
+    <row r="181" spans="1:4" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A181" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="C170" s="24">
+      <c r="C181" s="24">
         <v>0.19791666666666666</v>
       </c>
-      <c r="D170" s="24">
+      <c r="D181" s="24">
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="172" spans="1:5" ht="54" x14ac:dyDescent="0.25">
-      <c r="A172" s="33" t="s">
+    <row r="183" spans="1:4" ht="54" x14ac:dyDescent="0.25">
+      <c r="A183" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="C172" s="24">
+      <c r="C183" s="24">
         <v>0.25347222222222221</v>
       </c>
-      <c r="D172" s="24">
+      <c r="D183" s="24">
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A174" s="1" t="s">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A185" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C174" s="24">
+      <c r="C185" s="24">
         <v>0.11458333333333333</v>
       </c>
-      <c r="D174" s="24">
+      <c r="D185" s="24">
         <v>0.25</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A176" s="1" t="s">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A187" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C176" s="24">
+      <c r="C187" s="24">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="D176" s="24">
+      <c r="D187" s="24">
         <v>0.20833333333333334</v>
       </c>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A178" s="1" t="s">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A189" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C178" s="34">
-        <f>C180 - SUM(C158:C176)</f>
+      <c r="C189" s="34">
+        <f>C191 - SUM(C169:C187)</f>
         <v>0.71388888888888857</v>
       </c>
-      <c r="D178" s="48">
+      <c r="D189" s="36">
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A180" s="1" t="s">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A191" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C180" s="34">
+      <c r="C191" s="34">
         <v>3.3194444444444446</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="35">
+    <mergeCell ref="B125:B134"/>
+    <mergeCell ref="B136:B145"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="B55:B66"/>
+    <mergeCell ref="B157:E157"/>
+    <mergeCell ref="A158:B158"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:B83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B85:B92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B147:B156"/>
+    <mergeCell ref="B94:B102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B104:B112"/>
+    <mergeCell ref="B113:E113"/>
+    <mergeCell ref="B114:B123"/>
+    <mergeCell ref="B124:E124"/>
     <mergeCell ref="B135:E135"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -3438,29 +3562,12 @@
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B46:B53"/>
     <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:B66"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="A147:B147"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:B83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B85:B92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B136:B145"/>
-    <mergeCell ref="B94:B102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B104:B112"/>
-    <mergeCell ref="B113:E113"/>
-    <mergeCell ref="B114:B123"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="B125:B134"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C136:C145 C19:C27 C94:C102 C104:C112 C114:C123 C125:C134" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C85:C92 C74:C83 C55:C66 C68:C72 C29:C33 B6 C6:C17 C35:C44 C46:C53 C147:C156 C19:C27 C94:C102 C104:C112 C114:C123 C125:C134 C136:C145" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B136:B145 B94:B102 B104:B112 B114:B123 B125:B134" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B19:B27 B29:B33 B35:B44 B46:B53 B55:B66 B68:B72 B74:B83 B85:B92 B147:B156 B94:B102 B104:B112 B114:B123 B125:B134 B136:B145" xr:uid="{7694F886-C01B-440C-B6C8-5FF698F43C26}">
       <formula1>45261</formula1>
     </dataValidation>
   </dataValidations>
@@ -3469,7 +3576,7 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="23" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="22" orientation="portrait" r:id="rId2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -3664,15 +3771,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -3834,6 +3932,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
@@ -3851,14 +3958,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3874,4 +3973,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>